<commit_message>
Add ai_detailed data to XLSX (summary + domain + country)
</commit_message>
<xml_diff>
--- a/public/data/digest_combined_2026-05-06.xlsx
+++ b/public/data/digest_combined_2026-05-06.xlsx
@@ -587,7 +587,11 @@
           <t>Ормузька протока стала зброєю у геополітичному конфлікті</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Ормузька протока стала зброєю у геополітичному конфлікті Домен: логістика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -645,7 +649,11 @@
           <t>Трамп припинив супровід кораблів через Ормузьку протоку</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Трамп припинив супровід кораблів через Ормузьку протоку Домен: логістика Країна: США, Іран, Пакистан</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -703,7 +711,11 @@
           <t>Ринок нафти недооцінює дефіцит пропозиції з Близького Сходу</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Ринок нафти недооцінює дефіцит пропозиції з Близького Сходу Домен: енергетика Країна: Близький Схід</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -761,7 +773,11 @@
           <t>Бензин у США на 50% дорожче через іранську кризу</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Бензин у США на 50% дорожче через іранську кризу Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -819,7 +835,11 @@
           <t>Нова атака в Ормузькій протоці підкреслює ризики логістики</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Нова атака в Ормузькій протоці підкреслює ризики логістики Домен: геополітика Країна: Ормузька протока</t>
+        </is>
+      </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -877,7 +897,11 @@
           <t>США та союзники загрожують санкціями Ірану за Ормузьку протоку</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>США та союзники загрожують санкціями Ірану за Ормузьку протоку Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -931,7 +955,11 @@
           <t>Блокада США та закриття Ормузької протоки спричинили дефіцит нафти</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Блокада США та закриття Ормузької протоки спричинили дефіцит нафти Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -989,7 +1017,11 @@
           <t>США блокують Ормузький пролив для безпеки суден</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>США блокують Ормузький пролив для безпеки суден Домен: геополітика Країна: США</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1047,7 +1079,11 @@
           <t>Конфлікт США-Іран у Ормузькій протоці загрожує війною</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Конфлікт США-Іран у Ормузькій протоці загрожує війною Домен: геополітика Країна: США, Іран</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1105,7 +1141,11 @@
           <t>Іран атакує ОАЕ, загроза Ормузькій протоці</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Іран атакує ОАЕ, загроза Ормузькій протоці Домен: геополітика Країна: Іран, ОАЕ</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1163,7 +1203,11 @@
           <t>РФ атакує газовидобуток, ВВП України скорочується</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>РФ атакує газовидобуток, ВВП України скорочується Домен: геополітика Країна: Україна</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1221,7 +1265,11 @@
           <t>Удари РФ змушують Нафтогаз імпортувати більше газу</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Удари РФ змушують Нафтогаз імпортувати більше газу Домен: енергетика Країна: Україна</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -1279,7 +1327,11 @@
           <t>США та Бахрейн підтримують резолюцію ООН про санкції Іраніу</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>США та Бахрейн підтримують резолюцію ООН про санкції Іраніу Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1333,7 +1385,11 @@
           <t>Росія захопила частку аграрного гіганта</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Росія захопила частку аграрного гіганта Домен: геополітика Країна: Росія</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1391,7 +1447,11 @@
           <t>Кораблі кластеризуються біля Дубая через Іран</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Кораблі кластеризуються біля Дубая через Іран Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1449,7 +1509,11 @@
           <t>Атака дронів зупинила Кіришський НПЗ Росії</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Атака дронів зупинила Кіришський НПЗ Росії Домен: геополітика Країна: Росія</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1507,7 +1571,11 @@
           <t>Близькосхідна криза піднімає ціни нафти на 2027 рік</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Близькосхідна криза піднімає ціни нафти на 2027 рік Домен: геополітика Країна: США, Іран, країни Перської затоки</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1565,7 +1633,11 @@
           <t>Офіційний курс євро знизився на 6 копійок до 51,39 грн</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Офіційний курс євро знизився на 6 копійок до 51,39 грн Домен: валюта_фінанси Країна: Україна</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -1619,7 +1691,11 @@
           <t>MSC запускає нову лінію обходячи Ормузьку протоку</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>MSC запускає нову лінію обходячи Ормузьку протоку Домен: логістика Країна: Перс. затока</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -1677,7 +1753,11 @@
           <t>ОАЕ обмежує повітряний простір після іранської атаки</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>ОАЕ обмежує повітряний простір після іранської атаки Домен: геополітика Країна: ОАЕ</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1731,7 +1811,11 @@
           <t>Іранська ракета влучила в судно HMM у Перській затоці</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Іранська ракета влучила в судно HMM у Перській затоці Домен: геополітика Країна: ОАЕ, Іран</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1785,7 +1869,11 @@
           <t>Audi попереджає про значний вплив тарифів Трампа</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Audi попереджає про значний вплив тарифів Трампа Домен: санкції_торгівля Країна: США, Німеччина</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -1843,7 +1931,11 @@
           <t>США та Іран обмінюються вогнем у Перській затоці</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>США та Іран обмінюються вогнем у Перській затоці Домен: геополітика Країна: США, Іран</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -1897,7 +1989,11 @@
           <t>Конфлікт Іран-Ізраїль загрожує енергетичним шоком Європі</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Конфлікт Іран-Ізраїль загрожує енергетичним шоком Європі Домен: енергетика Країна: Іран, Ізраїль, Європа</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -1955,7 +2051,11 @@
           <t>Індійські акції падають, рупія на мінімумі через нафту</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Індійські акції падають, рупія на мінімумі через нафту Домен: енергетика Країна: Індія</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -2013,7 +2113,11 @@
           <t>Південнокорейське судно горить у Ормузькій протоці</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Південнокорейське судно горить у Ормузькій протоці Домен: логістика Країна: Іран, Південна Корея</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -2067,7 +2171,11 @@
           <t>Російські ракети вбили семеро в Харківській області</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Російські ракети вбили семеро в Харківській області Домен: геополітика Країна: Україна</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -2121,7 +2229,11 @@
           <t>США планують підвищити мита на автомобілі ЄС</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>США планують підвищити мита на автомобілі ЄС Домен: санкції_торгівля Країна: США, ЄС</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -2179,7 +2291,11 @@
           <t>Судно Maersk виходить з Перської затоки під охороною США</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Судно Maersk виходить з Перської затоки під охороною США Домен: геополітика Країна: Іран, США</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -2237,7 +2353,11 @@
           <t>Chevron стурбована транзитом через Гормуз на тлі конфлікту США-Іран</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Chevron стурбована транзитом через Гормуз на тлі конфлікту США-Іран Домен: геополітика Країна: США, Іран</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -2295,7 +2415,11 @@
           <t>Кораблі відступають через розширення контролю Іраном Ормузької протоки</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Кораблі відступають через розширення контролю Іраном Ормузької протоки Домен: логістика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -2349,7 +2473,11 @@
           <t>Пожежа на нафтовому комплексі Fujairah після атаки дронів</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Пожежа на нафтовому комплексі Fujairah після атаки дронів Домен: геополітика Країна: ОАЕ, Іран</t>
+        </is>
+      </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -2407,7 +2535,11 @@
           <t>Німецькі автовиробники в центрі тарифної атаки Трампа</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Німецькі автовиробники в центрі тарифної атаки Трампа Домен: санкції_торгівля Країна: США, Німеччина</t>
+        </is>
+      </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -2465,7 +2597,11 @@
           <t>Судноплавство в Ормузькій протоці паралізовано</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Судноплавство в Ормузькій протоці паралізовано Домен: логістика Країна: Іран, ОАЕ, Саудівська Аравія</t>
+        </is>
+      </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -2523,7 +2659,11 @@
           <t>Іран блокує американські військові кораблі в Ормузькій протоці</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Іран блокує американські військові кораблі в Ормузькій протоці Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -2581,7 +2721,11 @@
           <t>Сухогруз атакований біля Ірану, загроза логістиці</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Сухогруз атакований біля Ірану, загроза логістиці Домен: логістика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -2635,7 +2779,11 @@
           <t>Українські дрони вдарили по портовому комплексу Приморськ</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Українські дрони вдарили по портовому комплексу Приморськ Домен: логістика Країна: Росія</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -2693,7 +2841,11 @@
           <t>Іран та Китай проводять дипломатичні переговори в Пекіні</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr"/>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Іран та Китай проводять дипломатичні переговори в Пекіні Домен: геополітика Країна: Іран, Китай, США</t>
+        </is>
+      </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -2747,7 +2899,11 @@
           <t>Українське місто Олешки відрізане від поставок місяцями</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr"/>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Українське місто Олешки відрізане від поставок місяцями Домен: логістика Країна: Україна</t>
+        </is>
+      </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -2805,7 +2961,11 @@
           <t>Іранський дипломат вперше відвідує Китай після конфлікту</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr"/>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Іранський дипломат вперше відвідує Китай після конфлікту Домен: геополітика Країна: Іран, Китай</t>
+        </is>
+      </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -2859,7 +3019,11 @@
           <t>Китай та Іран проводять переговори на тлі паузи США</t>
         </is>
       </c>
-      <c r="F42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Китай та Іран проводять переговори на тлі паузи США Домен: геополітика Країна: Китай, Іран, США</t>
+        </is>
+      </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -2913,7 +3077,11 @@
           <t>Росія завдає ударів в Україні перед перемир'ям</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr"/>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Росія завдає ударів в Україні перед перемир'ям Домен: геополітика Країна: Україна, Росія</t>
+        </is>
+      </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -2967,7 +3135,11 @@
           <t>Трамп призупиняє операцію Hormuz на переговорах з Іраном</t>
         </is>
       </c>
-      <c r="F44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Трамп призупиняє операцію Hormuz на переговорах з Іраном Домен: геополітика Країна: Іран, США</t>
+        </is>
+      </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -3025,7 +3197,11 @@
           <t>Нафта падає на сигналах можливої угоди з Іраном</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Нафта падає на сигналах можливої угоди з Іраном Домен: енергетика Країна: Іран, США</t>
+        </is>
+      </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -3083,7 +3259,11 @@
           <t>ДРК переходить з кобальту на мідь через ціни</t>
         </is>
       </c>
-      <c r="F46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>ДРК переходить з кобальту на мідь через ціни Домен: ціни_сировини Країна: Демократична Республіка Конго</t>
+        </is>
+      </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -3141,7 +3321,11 @@
           <t>Occidental скорочує видобуток через іранський конфлікт</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr"/>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Occidental скорочує видобуток через іранський конфлікт Домен: геополітика Країна: США, Іран</t>
+        </is>
+      </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -3199,7 +3383,11 @@
           <t>Американський хімічний танкер вийшов з Ормузької протоки</t>
         </is>
       </c>
-      <c r="F48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Американський хімічний танкер вийшов з Ормузької протоки Домен: геополітика Країна: США, Ормузька протока</t>
+        </is>
+      </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -3257,7 +3445,11 @@
           <t>CENTCOM забезпечує безпечні маршрути через Ормузьку протоку</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr"/>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>CENTCOM забезпечує безпечні маршрути через Ормузьку протоку Домен: геополітика Країна: США</t>
+        </is>
+      </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -3311,7 +3503,11 @@
           <t>ОАЕ вийшла з ОПЕК, ослабивши картель</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>ОАЕ вийшла з ОПЕК, ослабивши картель Домен: геополітика Країна: ОАЕ</t>
+        </is>
+      </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -3369,7 +3565,11 @@
           <t>Російський танкер застряг біля Куби через блокаду США</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr"/>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Російський танкер застряг біля Куби через блокаду США Домен: санкції_торгівля Країна: Куба</t>
+        </is>
+      </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -3427,7 +3627,11 @@
           <t>Розпад ОПЕК загрожує енергетичною волатильністю</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr"/>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Розпад ОПЕК загрожує енергетичною волатильністю Домен: геополітика</t>
+        </is>
+      </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -3481,7 +3685,11 @@
           <t>США підвищують тарифи на авто ЄС до 25%</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr"/>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>США підвищують тарифи на авто ЄС до 25% Домен: санкції_торгівля Країна: ЄС</t>
+        </is>
+      </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -3539,7 +3747,11 @@
           <t>Рубіо заявляє про оборонний характер операцій США в Ормузі</t>
         </is>
       </c>
-      <c r="F54" s="5" t="inlineStr"/>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Рубіо заявляє про оборонний характер операцій США в Ормузі Домен: геополітика Країна: США, Іран</t>
+        </is>
+      </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -3597,7 +3809,11 @@
           <t>Ціни на нафту впали на 3% при відновленні проходу Ормузу</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr"/>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Ціни на нафту впали на 3% при відновленні проходу Ормузу Домен: ціни_сировини Країна: США, Іран</t>
+        </is>
+      </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -3655,7 +3871,11 @@
           <t>Пентагон відновлює Ормузьку протоку, але з обмеженнями</t>
         </is>
       </c>
-      <c r="F56" s="5" t="inlineStr"/>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Пентагон відновлює Ормузьку протоку, але з обмеженнями Домен: логістика Країна: США</t>
+        </is>
+      </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -3709,7 +3929,11 @@
           <t>Сенатори США вимагають повернути санкції на російну нафту</t>
         </is>
       </c>
-      <c r="F57" s="5" t="inlineStr"/>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Сенатори США вимагають повернути санкції на російну нафту Домен: санкції_торгівля Країна: Росія, США</t>
+        </is>
+      </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -3767,7 +3991,11 @@
           <t>Іранська напруженість підвищує маржі нафторафінування</t>
         </is>
       </c>
-      <c r="F58" s="5" t="inlineStr"/>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Іранська напруженість підвищує маржі нафторафінування Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -3825,7 +4053,11 @@
           <t>Diamondback додає 10% буріння в Permian через іранську напруженість</t>
         </is>
       </c>
-      <c r="F59" s="5" t="inlineStr"/>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Diamondback додає 10% буріння в Permian через іранську напруженість Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -3883,7 +4115,11 @@
           <t>QatarEnergy продовжує force majeure на LNG до липня</t>
         </is>
       </c>
-      <c r="F60" s="5" t="inlineStr"/>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>QatarEnergy продовжує force majeure на LNG до липня Домен: енергетика Країна: Катар</t>
+        </is>
+      </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -3941,7 +4177,11 @@
           <t>Макрон про марнування часу на тарифні загрози</t>
         </is>
       </c>
-      <c r="F61" s="5" t="inlineStr"/>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>Макрон про марнування часу на тарифні загрози Домен: санкції_торгівля Країна: США, ЄС, Німеччина</t>
+        </is>
+      </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -3995,7 +4235,11 @@
           <t>Ізраїльська компанія припиняє закупівлі російського зерна</t>
         </is>
       </c>
-      <c r="F62" s="5" t="inlineStr"/>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>Ізраїльська компанія припиняє закупівлі російського зерна Домен: санкції_торгівля Країна: Ізраїль, Росія, Україна</t>
+        </is>
+      </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -4053,7 +4297,11 @@
           <t>G7 координує дії щодо критичних мінералів проти Китаю</t>
         </is>
       </c>
-      <c r="F63" s="5" t="inlineStr"/>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>G7 координує дії щодо критичних мінералів проти Китаю Домен: санкції_торгівля Країна: Франція, Китай</t>
+        </is>
+      </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -4111,7 +4359,11 @@
           <t>Росія збільшує експорт нафти на максимумі часів війни</t>
         </is>
       </c>
-      <c r="F64" s="5" t="inlineStr"/>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Росія збільшує експорт нафти на максимумі часів війни Домен: ціни_сировини Країна: Росія</t>
+        </is>
+      </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -4169,7 +4421,11 @@
           <t>Танкерна компанія Bruton зафіксувала довгостроковий чартер</t>
         </is>
       </c>
-      <c r="F65" s="5" t="inlineStr"/>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Танкерна компанія Bruton зафіксувала довгостроковий чартер Домен: логістика Країна: Китай</t>
+        </is>
+      </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -4227,7 +4483,11 @@
           <t>ЕЦБ закликає Європу зменшити залежність від енергоімпорту</t>
         </is>
       </c>
-      <c r="F66" s="5" t="inlineStr"/>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>ЕЦБ закликає Європу зменшити залежність від енергоімпорту Домен: енергетика Країна: Європа</t>
+        </is>
+      </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -4285,7 +4545,11 @@
           <t>Українські дрони атакують на 1600 км в глибину Росії</t>
         </is>
       </c>
-      <c r="F67" s="5" t="inlineStr"/>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Українські дрони атакують на 1600 км в глибину Росії Домен: геополітика Країна: Україна, Росія</t>
+        </is>
+      </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -4339,7 +4603,11 @@
           <t>Конфлікт США-Іран у Перській затоці ризикує перерости в війну</t>
         </is>
       </c>
-      <c r="F68" s="5" t="inlineStr"/>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Конфлікт США-Іран у Перській затоці ризикує перерости в війну Домен: геополітика Країна: Іран, США</t>
+        </is>
+      </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -4393,7 +4661,11 @@
           <t>Запаси бензину США падають до історичних мінімумів</t>
         </is>
       </c>
-      <c r="F69" s="5" t="inlineStr"/>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Запаси бензину США падають до історичних мінімумів Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -4451,7 +4723,11 @@
           <t>Ціни на яловичину залишатимуться високими</t>
         </is>
       </c>
-      <c r="F70" s="5" t="inlineStr"/>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Ціни на яловичину залишатимуться високими Домен: ціни_сировини Країна: США</t>
+        </is>
+      </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -4509,7 +4785,11 @@
           <t>Китайські рафінерії готуються до санкцій проти Ірану</t>
         </is>
       </c>
-      <c r="F71" s="5" t="inlineStr"/>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>Китайські рафінерії готуються до санкцій проти Ірану Домен: санкції_торгівля Країна: Китай, Іран</t>
+        </is>
+      </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -4567,7 +4847,11 @@
           <t>США намагаються відкрити Ормузьку протоку під атаками</t>
         </is>
       </c>
-      <c r="F72" s="5" t="inlineStr"/>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>США намагаються відкрити Ормузьку протоку під атаками Домен: геополітика Країна: США, ОАЕ, Іран</t>
+        </is>
+      </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -4625,7 +4909,11 @@
           <t>Ризик перезапуску іранської війни залишається високим</t>
         </is>
       </c>
-      <c r="F73" s="5" t="inlineStr"/>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Ризик перезапуску іранської війни залишається високим Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -4683,7 +4971,11 @@
           <t>Акції Перської затоки падають після нових атак</t>
         </is>
       </c>
-      <c r="F74" s="5" t="inlineStr"/>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>Акції Перської затоки падають після нових атак Домен: геополітика Країна: ОАЕ, Іран</t>
+        </is>
+      </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -4741,7 +5033,11 @@
           <t>Трамп дестабілізував OPEC, наслідки для енергоринку</t>
         </is>
       </c>
-      <c r="F75" s="5" t="inlineStr"/>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>Трамп дестабілізував OPEC, наслідки для енергоринку Домен: геополітика Країна: США</t>
+        </is>
+      </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -4799,7 +5095,11 @@
           <t>Конфлікт Іран-Ізраїль підвищує ціни на вугіль</t>
         </is>
       </c>
-      <c r="F76" s="5" t="inlineStr"/>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Конфлікт Іран-Ізраїль підвищує ціни на вугіль Домен: енергетика Країна: Іран, Ізраїль</t>
+        </is>
+      </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -4857,7 +5157,11 @@
           <t>Вибух на кораблі в Ормузькій протоці, Сеул розглядає план</t>
         </is>
       </c>
-      <c r="F77" s="5" t="inlineStr"/>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Вибух на кораблі в Ормузькій протоці, Сеул розглядає план Домен: логістика Країна: Південна Корея, США, Іран</t>
+        </is>
+      </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -4911,7 +5215,11 @@
           <t>Рупія впала до історичного мінімуму через конфлікт</t>
         </is>
       </c>
-      <c r="F78" s="5" t="inlineStr"/>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Рупія впала до історичного мінімуму через конфлікт Домен: валюта_фінанси Країна: Індія</t>
+        </is>
+      </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -4965,7 +5273,11 @@
           <t>Ціни на нафту зростають, облігації під тиском</t>
         </is>
       </c>
-      <c r="F79" s="5" t="inlineStr"/>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>Ціни на нафту зростають, облігації під тиском Домен: енергетика Країна: глобально</t>
+        </is>
+      </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -5023,7 +5335,11 @@
           <t>Дрон пошкодив обладнання на Запоріжській АЕС</t>
         </is>
       </c>
-      <c r="F80" s="5" t="inlineStr"/>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Дрон пошкодив обладнання на Запоріжській АЕС Домен: енергетика Країна: Україна</t>
+        </is>
+      </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -5077,7 +5393,11 @@
           <t>Повернення мит почнеться з 12 травня</t>
         </is>
       </c>
-      <c r="F81" s="5" t="inlineStr"/>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Повернення мит почнеться з 12 травня Домен: санкції_торгівля Країна: США</t>
+        </is>
+      </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -5131,7 +5451,11 @@
           <t>Азія стикається з енергокризою через іранський конфлікт</t>
         </is>
       </c>
-      <c r="F82" s="5" t="inlineStr"/>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Азія стикається з енергокризою через іранський конфлікт Домен: енергетика Країна: Азія</t>
+        </is>
+      </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -5189,7 +5513,11 @@
           <t>МВФ попереджає про гірші наслідки конфлікту на Близькому Сході</t>
         </is>
       </c>
-      <c r="F83" s="5" t="inlineStr"/>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>МВФ попереджає про гірші наслідки конфлікту на Близькому Сході Домен: геополітика Країна: Близький Схід</t>
+        </is>
+      </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -5243,7 +5571,11 @@
           <t>Судно Maersk транзитує Ормузький протоку з військовим супроводом</t>
         </is>
       </c>
-      <c r="F84" s="5" t="inlineStr"/>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Судно Maersk транзитує Ормузький протоку з військовим супроводом Домен: логістика Країна: ОАЕ, США</t>
+        </is>
+      </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -5297,7 +5629,11 @@
           <t>Chevron попереджає про наближаючийся дефіцит нафти</t>
         </is>
       </c>
-      <c r="F85" s="5" t="inlineStr"/>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Chevron попереджає про наближаючийся дефіцит нафти Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -5355,7 +5691,11 @@
           <t>Український дрон вдарив по московській висотці перед Днем Перемоги</t>
         </is>
       </c>
-      <c r="F86" s="5" t="inlineStr"/>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Український дрон вдарив по московській висотці перед Днем Перемоги Домен: геополітика Країна: Україна, Росія</t>
+        </is>
+      </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -5409,7 +5749,11 @@
           <t>Світові запаси нафти на мінімумі за 8 років</t>
         </is>
       </c>
-      <c r="F87" s="5" t="inlineStr"/>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Світові запаси нафти на мінімумі за 8 років Домен: енергетика</t>
+        </is>
+      </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -5463,7 +5807,11 @@
           <t>AI-бум збільшить вартість електроенергії на північному сході США</t>
         </is>
       </c>
-      <c r="F88" s="5" t="inlineStr"/>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>AI-бум збільшить вартість електроенергії на північному сході США Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -5521,7 +5869,11 @@
           <t>Amazon запустив послугу логістики, акції перевізників впали</t>
         </is>
       </c>
-      <c r="F89" s="5" t="inlineStr"/>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Amazon запустив послугу логістики, акції перевізників впали Домен: логістика Країна: США</t>
+        </is>
+      </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -5575,7 +5927,11 @@
           <t>Іранська криза може спричинити стрибок цін на добрива</t>
         </is>
       </c>
-      <c r="F90" s="5" t="inlineStr"/>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Іранська криза може спричинити стрибок цін на добрива Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -5633,7 +5989,11 @@
           <t>Росія інтенсифікує атаки дронів на портали України</t>
         </is>
       </c>
-      <c r="F91" s="5" t="inlineStr"/>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Росія інтенсифікує атаки дронів на портали України Домен: логістика Країна: Україна, Росія</t>
+        </is>
+      </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -5687,7 +6047,11 @@
           <t>Китай вводить санкції проти США щодо нафторозпилювачів</t>
         </is>
       </c>
-      <c r="F92" s="5" t="inlineStr"/>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>Китай вводить санкції проти США щодо нафторозпилювачів Домен: санкції_торгівля Країна: Китай, США</t>
+        </is>
+      </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -5745,7 +6109,11 @@
           <t>Доларизація та падіння європейських ринків</t>
         </is>
       </c>
-      <c r="F93" s="5" t="inlineStr"/>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>Доларизація та падіння європейських ринків Домен: валюта_фінанси Країна: США, ЄС</t>
+        </is>
+      </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -5799,7 +6167,11 @@
           <t>Німецькі автовиробники занепокоєні Близькосхідною кризою</t>
         </is>
       </c>
-      <c r="F94" s="5" t="inlineStr"/>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Німецькі автовиробники занепокоєні Близькосхідною кризою Домен: геополітика Країна: Німеччина, Близький Схід</t>
+        </is>
+      </c>
       <c r="G94" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -5853,7 +6225,11 @@
           <t>ЄС готується до торговельних переговорів з США</t>
         </is>
       </c>
-      <c r="F95" s="5" t="inlineStr"/>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>ЄС готується до торговельних переговорів з США Домен: санкції_торгівля Країна: ЄС</t>
+        </is>
+      </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -5907,7 +6283,11 @@
           <t>Інвестори готуються до можливого нафтового шоку</t>
         </is>
       </c>
-      <c r="F96" s="5" t="inlineStr"/>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>Інвестори готуються до можливого нафтового шоку Домен: енергетика</t>
+        </is>
+      </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -5961,7 +6341,11 @@
           <t>Авіалінії підвищують ціни через зростання вартості палива</t>
         </is>
       </c>
-      <c r="F97" s="5" t="inlineStr"/>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>Авіалінії підвищують ціни через зростання вартості палива Домен: енергетика Країна: світ</t>
+        </is>
+      </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -6019,7 +6403,11 @@
           <t>Атака на танкер у Ормузькій протоці загрожує логістиці</t>
         </is>
       </c>
-      <c r="F98" s="5" t="inlineStr"/>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>Атака на танкер у Ормузькій протоці загрожує логістиці Домен: логістика Країна: ОАЕ, Іран</t>
+        </is>
+      </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -6077,7 +6465,11 @@
           <t>Отрута в дитячому харчуванні в Австрії</t>
         </is>
       </c>
-      <c r="F99" s="5" t="inlineStr"/>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>Отрута в дитячому харчуванні в Австрії Домен: здоров'я_біобезпека Країна: Австрія</t>
+        </is>
+      </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
           <t>здоров'я_біобезпека</t>
@@ -6135,7 +6527,11 @@
           <t>США задушують іранську нафтову промисловість</t>
         </is>
       </c>
-      <c r="F100" s="5" t="inlineStr"/>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>США задушують іранську нафтову промисловість Домен: енергетика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -6193,7 +6589,11 @@
           <t>США — постачальник нафти останньої надії при збоях у Ормузі</t>
         </is>
       </c>
-      <c r="F101" s="5" t="inlineStr"/>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>США — постачальник нафти останньої надії при збоях у Ормузі Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -6251,7 +6651,11 @@
           <t>ОПЕК+ третій раз підвищує квоти видобутку нафти</t>
         </is>
       </c>
-      <c r="F102" s="5" t="inlineStr"/>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>ОПЕК+ третій раз підвищує квоти видобутку нафти Домен: енергетика Країна: ОПЕК+</t>
+        </is>
+      </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -6309,7 +6713,11 @@
           <t>Австралія інвестує $7 млрд у стратегічний паливний резерв</t>
         </is>
       </c>
-      <c r="F103" s="5" t="inlineStr"/>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>Австралія інвестує $7 млрд у стратегічний паливний резерв Домен: енергетика Країна: Австралія</t>
+        </is>
+      </c>
       <c r="G103" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -6367,7 +6775,11 @@
           <t>Китайський попит на метали зростає через близькосхідний конфлікт</t>
         </is>
       </c>
-      <c r="F104" s="5" t="inlineStr"/>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>Китайський попит на метали зростає через близькосхідний конфлікт Домен: геополітика Країна: Китай</t>
+        </is>
+      </c>
       <c r="G104" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -6425,7 +6837,11 @@
           <t>Долар слабшає на надіях угоди США-Іран</t>
         </is>
       </c>
-      <c r="F105" s="5" t="inlineStr"/>
+      <c r="F105" s="5" t="inlineStr">
+        <is>
+          <t>Долар слабшає на надіях угоди США-Іран Домен: валюта_фінанси Країна: США, Іран, Японія</t>
+        </is>
+      </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -6479,7 +6895,11 @@
           <t>Sentinel Midstream будує глибоководний експортний термінал нафти</t>
         </is>
       </c>
-      <c r="F106" s="5" t="inlineStr"/>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>Sentinel Midstream будує глибоководний експортний термінал нафти Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G106" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -6537,7 +6957,11 @@
           <t>Страйк транспортників у Болівії блокує дороги</t>
         </is>
       </c>
-      <c r="F107" s="5" t="inlineStr"/>
+      <c r="F107" s="5" t="inlineStr">
+        <is>
+          <t>Страйк транспортників у Болівії блокує дороги Домен: страйки_перебої Країна: Болівія</t>
+        </is>
+      </c>
       <c r="G107" s="5" t="inlineStr">
         <is>
           <t>страйки_перебої</t>
@@ -6591,7 +7015,11 @@
           <t>Ціни на бензин перевищили $4.50 за галон</t>
         </is>
       </c>
-      <c r="F108" s="5" t="inlineStr"/>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>Ціни на бензин перевищили $4.50 за галон Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G108" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -6649,7 +7077,11 @@
           <t>Matson розширює флот LNG-контейнерів на $1 млрд</t>
         </is>
       </c>
-      <c r="F109" s="5" t="inlineStr"/>
+      <c r="F109" s="5" t="inlineStr">
+        <is>
+          <t>Matson розширює флот LNG-контейнерів на $1 млрд Домен: логістика Країна: США</t>
+        </is>
+      </c>
       <c r="G109" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -6707,7 +7139,11 @@
           <t>США експортують рекордні обсяги нафти для заповнення дефіциту</t>
         </is>
       </c>
-      <c r="F110" s="5" t="inlineStr"/>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>США експортують рекордні обсяги нафти для заповнення дефіциту Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G110" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -6765,7 +7201,11 @@
           <t>Індекс вуглецевих кредитів суден зріс до €225/т CO₂</t>
         </is>
       </c>
-      <c r="F111" s="5" t="inlineStr"/>
+      <c r="F111" s="5" t="inlineStr">
+        <is>
+          <t>Індекс вуглецевих кредитів суден зріс до €225/т CO₂ Домен: санкції_торгівля</t>
+        </is>
+      </c>
       <c r="G111" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -6819,7 +7259,11 @@
           <t>IMO ввела нові екологічні вимоги для суден</t>
         </is>
       </c>
-      <c r="F112" s="5" t="inlineStr"/>
+      <c r="F112" s="5" t="inlineStr">
+        <is>
+          <t>IMO ввела нові екологічні вимоги для суден Домен: санкції_торгівля</t>
+        </is>
+      </c>
       <c r="G112" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -6873,7 +7317,11 @@
           <t>Венесуела збільшила експорт нафти на 14% до 1,23 млн барелів/день</t>
         </is>
       </c>
-      <c r="F113" s="5" t="inlineStr"/>
+      <c r="F113" s="5" t="inlineStr">
+        <is>
+          <t>Венесуела збільшила експорт нафти на 14% до 1,23 млн барелів/день Домен: ціни_сировини Країна: Венесуела</t>
+        </is>
+      </c>
       <c r="G113" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -6931,7 +7379,11 @@
           <t>Саудівська Аравія знижує ціни на Arab Light для Азії</t>
         </is>
       </c>
-      <c r="F114" s="5" t="inlineStr"/>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>Саудівська Аравія знижує ціни на Arab Light для Азії Домен: ціни_сировини Країна: Саудівська Аравія</t>
+        </is>
+      </c>
       <c r="G114" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -6989,7 +7441,11 @@
           <t>Норвегія запустила газове родовище Eirin для Європи</t>
         </is>
       </c>
-      <c r="F115" s="5" t="inlineStr"/>
+      <c r="F115" s="5" t="inlineStr">
+        <is>
+          <t>Норвегія запустила газове родовище Eirin для Європи Домен: енергетика Країна: Норвегія</t>
+        </is>
+      </c>
       <c r="G115" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -7047,7 +7503,11 @@
           <t>Трамп закликає Іран здатися у конфлікті</t>
         </is>
       </c>
-      <c r="F116" s="5" t="inlineStr"/>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>Трамп закликає Іран здатися у конфлікті Домен: геополітика Країна: США, Іран</t>
+        </is>
+      </c>
       <c r="G116" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -7105,7 +7565,11 @@
           <t>США знімають санкції з Еритреї для покращення логістики Червоного моря</t>
         </is>
       </c>
-      <c r="F117" s="5" t="inlineStr"/>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>США знімають санкції з Еритреї для покращення логістики Червоного моря Домен: геополітика Країна: Еритрея</t>
+        </is>
+      </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -7159,7 +7623,11 @@
           <t>Розслідування США щодо тарифів на надлишкові потужності</t>
         </is>
       </c>
-      <c r="F118" s="5" t="inlineStr"/>
+      <c r="F118" s="5" t="inlineStr">
+        <is>
+          <t>Розслідування США щодо тарифів на надлишкові потужності Домен: санкції_торгівля Країна: США</t>
+        </is>
+      </c>
       <c r="G118" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -7213,7 +7681,11 @@
           <t>Китай ігнорує санкції, постачальники шукають альтернативи</t>
         </is>
       </c>
-      <c r="F119" s="5" t="inlineStr"/>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>Китай ігнорує санкції, постачальники шукають альтернативи Домен: геополітика Країна: Китай</t>
+        </is>
+      </c>
       <c r="G119" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -7267,7 +7739,11 @@
           <t>ADB інвестує $12.5 млрд у мінерали проти Китаю</t>
         </is>
       </c>
-      <c r="F120" s="5" t="inlineStr"/>
+      <c r="F120" s="5" t="inlineStr">
+        <is>
+          <t>ADB інвестує $12.5 млрд у мінерали проти Китаю Домен: ціни_сировини Країна: Узбекистан, Китай</t>
+        </is>
+      </c>
       <c r="G120" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -7325,7 +7801,11 @@
           <t>Видобуток золота в Амазонії спричиняє забруднення ртуттю</t>
         </is>
       </c>
-      <c r="F121" s="5" t="inlineStr"/>
+      <c r="F121" s="5" t="inlineStr">
+        <is>
+          <t>Видобуток золота в Амазонії спричиняє забруднення ртуттю Домен: погода_клімат Країна: Бразилія</t>
+        </is>
+      </c>
       <c r="G121" s="5" t="inlineStr">
         <is>
           <t>погода_клімат</t>
@@ -7383,7 +7863,11 @@
           <t>Перемир'я з Іраном не закінчилось — загроза судноплавству</t>
         </is>
       </c>
-      <c r="F122" s="5" t="inlineStr"/>
+      <c r="F122" s="5" t="inlineStr">
+        <is>
+          <t>Перемир'я з Іраном не закінчилось — загроза судноплавству Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G122" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -7437,7 +7921,11 @@
           <t>Партія Тиграю відновлює уряд у Північній Ефіопії</t>
         </is>
       </c>
-      <c r="F123" s="5" t="inlineStr"/>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>Партія Тиграю відновлює уряд у Північній Ефіопії Домен: геополітика Країна: Ефіопія</t>
+        </is>
+      </c>
       <c r="G123" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -7495,7 +7983,11 @@
           <t>Аргентинська автопромислова індустрія страждає від реформ Мілея</t>
         </is>
       </c>
-      <c r="F124" s="5" t="inlineStr"/>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>Аргентинська автопромислова індустрія страждає від реформ Мілея Домен: валюта_фінанси Країна: Аргентина</t>
+        </is>
+      </c>
       <c r="G124" s="5" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -7553,7 +8045,11 @@
           <t>ЄС вимагає прийняти угоду з США до липня</t>
         </is>
       </c>
-      <c r="F125" s="5" t="inlineStr"/>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>ЄС вимагає прийняти угоду з США до липня Домен: санкції_торгівля Країна: США, ЄС</t>
+        </is>
+      </c>
       <c r="G125" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -7607,7 +8103,11 @@
           <t>BP розглядає вихід з Північного моря через податки</t>
         </is>
       </c>
-      <c r="F126" s="5" t="inlineStr"/>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>BP розглядає вихід з Північного моря через податки Домен: енергетика Країна: Великобританія</t>
+        </is>
+      </c>
       <c r="G126" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -7665,7 +8165,11 @@
           <t>Британські облігації досягли максимуму за 26 років</t>
         </is>
       </c>
-      <c r="F127" s="5" t="inlineStr"/>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>Британські облігації досягли максимуму за 26 років Домен: валюта_фінанси Країна: Великобританія</t>
+        </is>
+      </c>
       <c r="G127" s="5" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -7719,7 +8223,11 @@
           <t>Саудівська Аравія має найбільший дефіцит бюджету з 2018 року</t>
         </is>
       </c>
-      <c r="F128" s="5" t="inlineStr"/>
+      <c r="F128" s="5" t="inlineStr">
+        <is>
+          <t>Саудівська Аравія має найбільший дефіцит бюджету з 2018 року Домен: геополітика Країна: Саудівська Аравія</t>
+        </is>
+      </c>
       <c r="G128" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -7777,7 +8285,11 @@
           <t>Канада перейшла на профіцит торгівлі завдяки нафті та золоту</t>
         </is>
       </c>
-      <c r="F129" s="5" t="inlineStr"/>
+      <c r="F129" s="5" t="inlineStr">
+        <is>
+          <t>Канада перейшла на профіцит торгівлі завдяки нафті та золоту Домен: ціни_сировини Країна: Канада</t>
+        </is>
+      </c>
       <c r="G129" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -7835,7 +8347,11 @@
           <t>Apple розглядає Intel та Samsung для виробництва чипів у США</t>
         </is>
       </c>
-      <c r="F130" s="5" t="inlineStr"/>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>Apple розглядає Intel та Samsung для виробництва чипів у США Домен: санкції_торгівля Країна: США</t>
+        </is>
+      </c>
       <c r="G130" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -7893,7 +8409,11 @@
           <t>Німецький експорт стагнує через невизначеність на Близькому Сході</t>
         </is>
       </c>
-      <c r="F131" s="5" t="inlineStr"/>
+      <c r="F131" s="5" t="inlineStr">
+        <is>
+          <t>Німецький експорт стагнує через невизначеність на Близькому Сході Домен: геополітика Країна: Німеччина</t>
+        </is>
+      </c>
       <c r="G131" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -7947,7 +8467,11 @@
           <t>Мозамбік переживає поглиблення фінансової кризи</t>
         </is>
       </c>
-      <c r="F132" s="5" t="inlineStr"/>
+      <c r="F132" s="5" t="inlineStr">
+        <is>
+          <t>Мозамбік переживає поглиблення фінансової кризи Домен: геополітика Країна: Мозамбік</t>
+        </is>
+      </c>
       <c r="G132" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -8001,7 +8525,11 @@
           <t>Авіавантажний ринок стабілізується, перепозиціонування потужностей</t>
         </is>
       </c>
-      <c r="F133" s="5" t="inlineStr"/>
+      <c r="F133" s="5" t="inlineStr">
+        <is>
+          <t>Авіавантажний ринок стабілізується, перепозиціонування потужностей Домен: логістика</t>
+        </is>
+      </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -8055,7 +8583,11 @@
           <t>Hapag-Lloyd пропонує наземну логістику до Перської затоки</t>
         </is>
       </c>
-      <c r="F134" s="5" t="inlineStr"/>
+      <c r="F134" s="5" t="inlineStr">
+        <is>
+          <t>Hapag-Lloyd пропонує наземну логістику до Перської затоки Домен: логістика Країна: ОАЕ, Кувейт, Саудівська Аравія, Катар, Ірак</t>
+        </is>
+      </c>
       <c r="G134" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -8113,7 +8645,11 @@
           <t>ЄС виявив зростання порушень щодо пестицидів</t>
         </is>
       </c>
-      <c r="F135" s="5" t="inlineStr"/>
+      <c r="F135" s="5" t="inlineStr">
+        <is>
+          <t>ЄС виявив зростання порушень щодо пестицидів Домен: митниця_регуляторика Країна: ЄС</t>
+        </is>
+      </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
           <t>митниця_регуляторика</t>
@@ -8171,7 +8707,11 @@
           <t>Ірак пропонує нафту з глибокими знижками</t>
         </is>
       </c>
-      <c r="F136" s="5" t="inlineStr"/>
+      <c r="F136" s="5" t="inlineStr">
+        <is>
+          <t>Ірак пропонує нафту з глибокими знижками Домен: логістика Країна: Ірак</t>
+        </is>
+      </c>
       <c r="G136" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -8229,7 +8769,11 @@
           <t>Російський LNG зріс на 8.6% у січні-квітні</t>
         </is>
       </c>
-      <c r="F137" s="5" t="inlineStr"/>
+      <c r="F137" s="5" t="inlineStr">
+        <is>
+          <t>Російський LNG зріс на 8.6% у січні-квітні Домен: енергетика Країна: Росія</t>
+        </is>
+      </c>
       <c r="G137" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -8287,7 +8831,11 @@
           <t>Ірак знижує ціни на нафту для перевезення через Ормузь</t>
         </is>
       </c>
-      <c r="F138" s="5" t="inlineStr"/>
+      <c r="F138" s="5" t="inlineStr">
+        <is>
+          <t>Ірак знижує ціни на нафту для перевезення через Ормузь Домен: енергетика Країна: Ірак</t>
+        </is>
+      </c>
       <c r="G138" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -8345,7 +8893,11 @@
           <t>Південноафриканський ранд падає через напруженість США-Іран</t>
         </is>
       </c>
-      <c r="F139" s="5" t="inlineStr"/>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>Південноафриканський ранд падає через напруженість США-Іран Домен: геополітика Країна: Південна Африка</t>
+        </is>
+      </c>
       <c r="G139" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -8399,7 +8951,11 @@
           <t>Експорт енергії США викликає занепокоєння через ціни на паливо</t>
         </is>
       </c>
-      <c r="F140" s="5" t="inlineStr"/>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>Експорт енергії США викликає занепокоєння через ціни на паливо Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G140" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -8457,7 +9013,11 @@
           <t>Україна атакує російський нафторафінерій Кіріші</t>
         </is>
       </c>
-      <c r="F141" s="5" t="inlineStr"/>
+      <c r="F141" s="5" t="inlineStr">
+        <is>
+          <t>Україна атакує російський нафторафінерій Кіріші Домен: геополітика Країна: Росія, Україна</t>
+        </is>
+      </c>
       <c r="G141" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -8515,7 +9075,11 @@
           <t>Вибух у колумбійській шахті вбив дев'ять робітників</t>
         </is>
       </c>
-      <c r="F142" s="5" t="inlineStr"/>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>Вибух у колумбійській шахті вбив дев'ять робітників Домен: логістика Країна: Колумбія</t>
+        </is>
+      </c>
       <c r="G142" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -8573,7 +9137,11 @@
           <t>Зростання приватного сектору ОАЕ сповільнюється через конфлікт</t>
         </is>
       </c>
-      <c r="F143" s="5" t="inlineStr"/>
+      <c r="F143" s="5" t="inlineStr">
+        <is>
+          <t>Зростання приватного сектору ОАЕ сповільнюється через конфлікт Домен: геополітика Країна: ОАЕ, Іран</t>
+        </is>
+      </c>
       <c r="G143" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -8627,7 +9195,11 @@
           <t>Долар слабшає на фоні близькосхідного перемир'я</t>
         </is>
       </c>
-      <c r="F144" s="5" t="inlineStr"/>
+      <c r="F144" s="5" t="inlineStr">
+        <is>
+          <t>Долар слабшає на фоні близькосхідного перемир'я Домен: валюта_фінанси</t>
+        </is>
+      </c>
       <c r="G144" s="5" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -8677,7 +9249,11 @@
           <t>Британські фірми витісняються з ЄС через червону стрічку</t>
         </is>
       </c>
-      <c r="F145" s="5" t="inlineStr"/>
+      <c r="F145" s="5" t="inlineStr">
+        <is>
+          <t>Британські фірми витісняються з ЄС через червону стрічку Домен: санкції_торгівля Країна: Великобританія, ЄС</t>
+        </is>
+      </c>
       <c r="G145" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -8731,7 +9307,11 @@
           <t>Іран завдав ударів по ОАЕ, Британія засуджує</t>
         </is>
       </c>
-      <c r="F146" s="5" t="inlineStr"/>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>Іран завдав ударів по ОАЕ, Британія засуджує Домен: геополітика Країна: ОАЕ, Іран</t>
+        </is>
+      </c>
       <c r="G146" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -8785,7 +9365,11 @@
           <t>США шукають підтримку Китаю та Південної Кореї в іранській кризі</t>
         </is>
       </c>
-      <c r="F147" s="5" t="inlineStr"/>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>США шукають підтримку Китаю та Південної Кореї в іранській кризі Домен: геополітика Країна: США, Китай, Південна Корея, Іран</t>
+        </is>
+      </c>
       <c r="G147" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -8839,7 +9423,11 @@
           <t>Amazon розширює власну логістику, FedEx і UPS втрачають акції</t>
         </is>
       </c>
-      <c r="F148" s="5" t="inlineStr"/>
+      <c r="F148" s="5" t="inlineStr">
+        <is>
+          <t>Amazon розширює власну логістику, FedEx і UPS втрачають акції Домен: логістика Країна: США</t>
+        </is>
+      </c>
       <c r="G148" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -8893,7 +9481,11 @@
           <t>Іранський конфлікт підвищує ціни на бензин, падають продажі ресторанів</t>
         </is>
       </c>
-      <c r="F149" s="5" t="inlineStr"/>
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>Іранський конфлікт підвищує ціни на бензин, падають продажі ресторанів Домен: енергетика Країна: США, Іран</t>
+        </is>
+      </c>
       <c r="G149" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -8951,7 +9543,11 @@
           <t>Росія оголошує перемир'я на День Перемоги, Київ раніше</t>
         </is>
       </c>
-      <c r="F150" s="5" t="inlineStr"/>
+      <c r="F150" s="5" t="inlineStr">
+        <is>
+          <t>Росія оголошує перемир'я на День Перемоги, Київ раніше Домен: геополітика Країна: Україна</t>
+        </is>
+      </c>
       <c r="G150" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -9005,7 +9601,11 @@
           <t>США продовжують захист венесуельської Citgo</t>
         </is>
       </c>
-      <c r="F151" s="5" t="inlineStr"/>
+      <c r="F151" s="5" t="inlineStr">
+        <is>
+          <t>США продовжують захист венесуельської Citgo Домен: санкції_торгівля Країна: Венесуела</t>
+        </is>
+      </c>
       <c r="G151" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -9063,7 +9663,11 @@
           <t>Соя росте на початку тижня</t>
         </is>
       </c>
-      <c r="F152" s="5" t="inlineStr"/>
+      <c r="F152" s="5" t="inlineStr">
+        <is>
+          <t>Соя росте на початку тижня Домен: ціни_сировини</t>
+        </is>
+      </c>
       <c r="G152" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -9117,7 +9721,11 @@
           <t>ЕЦБ може підняти ставки у червні — Нагель</t>
         </is>
       </c>
-      <c r="F153" s="5" t="inlineStr"/>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>ЕЦБ може підняти ставки у червні — Нагель Домен: валюта_фінанси Країна: Євросоюз</t>
+        </is>
+      </c>
       <c r="G153" s="5" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -9171,7 +9779,11 @@
           <t>Eni відновила видобуток нафти у Венесуелі у квітні</t>
         </is>
       </c>
-      <c r="F154" s="5" t="inlineStr"/>
+      <c r="F154" s="5" t="inlineStr">
+        <is>
+          <t>Eni відновила видобуток нафти у Венесуелі у квітні Домен: санкції_торгівля Країна: Венесуела, Італія</t>
+        </is>
+      </c>
       <c r="G154" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -9229,7 +9841,11 @@
           <t>Армія Судану звинувачує ОАЕ та Ефіопію в атаці дронів</t>
         </is>
       </c>
-      <c r="F155" s="5" t="inlineStr"/>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>Армія Судану звинувачує ОАЕ та Ефіопію в атаці дронів Домен: геополітика Країна: Судан, ОАЕ, Ефіопія</t>
+        </is>
+      </c>
       <c r="G155" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -9283,7 +9899,11 @@
           <t>Канада запускає програму допомоги від тарифів на 1 млрд</t>
         </is>
       </c>
-      <c r="F156" s="5" t="inlineStr"/>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
+          <t>Канада запускає програму допомоги від тарифів на 1 млрд Домен: санкції_торгівля Країна: Канада</t>
+        </is>
+      </c>
       <c r="G156" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -9337,7 +9957,11 @@
           <t>Південна Африка стикається з посухою El Niño та іранською кризою</t>
         </is>
       </c>
-      <c r="F157" s="5" t="inlineStr"/>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>Південна Африка стикається з посухою El Niño та іранською кризою Домен: погода_клімат Країна: Південна Африка, Іран</t>
+        </is>
+      </c>
       <c r="G157" s="5" t="inlineStr">
         <is>
           <t>погода_клімат</t>
@@ -9395,7 +10019,11 @@
           <t>Напруженість на Близькому Сході впливає на ринки</t>
         </is>
       </c>
-      <c r="F158" s="5" t="inlineStr"/>
+      <c r="F158" s="5" t="inlineStr">
+        <is>
+          <t>Напруженість на Близькому Сході впливає на ринки Домен: геополітика Країна: Близький Схід</t>
+        </is>
+      </c>
       <c r="G158" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -9453,7 +10081,11 @@
           <t>Спалах хантавірусу на судні біля Кабо-Верде</t>
         </is>
       </c>
-      <c r="F159" s="5" t="inlineStr"/>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>Спалах хантавірусу на судні біля Кабо-Верде Домен: здоров'я_біобезпека Країна: Кабо-Верде</t>
+        </is>
+      </c>
       <c r="G159" s="5" t="inlineStr">
         <is>
           <t>здоров'я_біобезпека</t>
@@ -9507,7 +10139,11 @@
           <t>Швеція арештувала китайського капітана судна, пов'язаного з Росією</t>
         </is>
       </c>
-      <c r="F160" s="5" t="inlineStr"/>
+      <c r="F160" s="5" t="inlineStr">
+        <is>
+          <t>Швеція арештувала китайського капітана судна, пов'язаного з Росією Домен: санкції_торгівля Країна: Швеція, Китай, Росія</t>
+        </is>
+      </c>
       <c r="G160" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -9561,7 +10197,11 @@
           <t>Швеція знижує залізничні збори на 20% з 2028 року</t>
         </is>
       </c>
-      <c r="F161" s="5" t="inlineStr"/>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>Швеція знижує залізничні збори на 20% з 2028 року Домен: логістика Країна: Швеція</t>
+        </is>
+      </c>
       <c r="G161" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -9615,7 +10255,11 @@
           <t>Дубай розширює операції після відновлення повітряного простору</t>
         </is>
       </c>
-      <c r="F162" s="5" t="inlineStr"/>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>Дубай розширює операції після відновлення повітряного простору Домен: логістика Країна: ОАЕ</t>
+        </is>
+      </c>
       <c r="G162" s="5" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -9669,7 +10313,11 @@
           <t>ФРС не знижуватиме ставки у 2026 році</t>
         </is>
       </c>
-      <c r="F163" s="5" t="inlineStr"/>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>ФРС не знижуватиме ставки у 2026 році Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G163" s="5" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -9723,7 +10371,11 @@
           <t>США готуються до повернення тарифів</t>
         </is>
       </c>
-      <c r="F164" s="5" t="inlineStr"/>
+      <c r="F164" s="5" t="inlineStr">
+        <is>
+          <t>США готуються до повернення тарифів Домен: санкції_торгівля Країна: США</t>
+        </is>
+      </c>
       <c r="G164" s="5" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -9777,7 +10429,11 @@
           <t>Резистентність до кокцидіозу вимагає оновлення програм лікування</t>
         </is>
       </c>
-      <c r="F165" s="5" t="inlineStr"/>
+      <c r="F165" s="5" t="inlineStr">
+        <is>
+          <t>Резистентність до кокцидіозу вимагає оновлення програм лікування Домен: здоров'я_біобезпека Країна: світ</t>
+        </is>
+      </c>
       <c r="G165" s="5" t="inlineStr">
         <is>
           <t>здоров'я_біобезпека</t>
@@ -9835,7 +10491,11 @@
           <t>Австралія та Японія посилюють співпрацю з критичних мінералів</t>
         </is>
       </c>
-      <c r="F166" s="5" t="inlineStr"/>
+      <c r="F166" s="5" t="inlineStr">
+        <is>
+          <t>Австралія та Японія посилюють співпрацю з критичних мінералів Домен: геополітика Країна: Австралія, Японія</t>
+        </is>
+      </c>
       <c r="G166" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -9893,7 +10553,11 @@
           <t>Індійське виробництво уповільнюється через військові витрати</t>
         </is>
       </c>
-      <c r="F167" s="5" t="inlineStr"/>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>Індійське виробництво уповільнюється через військові витрати Домен: ціни_сировини Країна: Індія</t>
+        </is>
+      </c>
       <c r="G167" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -9951,7 +10615,11 @@
           <t>Вартість кормів зростає, нові виклики в 2026 році</t>
         </is>
       </c>
-      <c r="F168" s="5" t="inlineStr"/>
+      <c r="F168" s="5" t="inlineStr">
+        <is>
+          <t>Вартість кормів зростає, нові виклики в 2026 році Домен: ціни_сировини</t>
+        </is>
+      </c>
       <c r="G168" s="5" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -10005,7 +10673,11 @@
           <t>ЄЦБ: ризики рецесії в єврозоні реальні та обґрунтовані</t>
         </is>
       </c>
-      <c r="F169" s="5" t="inlineStr"/>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>ЄЦБ: ризики рецесії в єврозоні реальні та обґрунтовані Домен: валюта_фінанси Країна: Євросоюз</t>
+        </is>
+      </c>
       <c r="G169" s="5" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -10059,7 +10731,11 @@
           <t>Невизначеність США-Іран обмежує зростання на Перській затоці</t>
         </is>
       </c>
-      <c r="F170" s="5" t="inlineStr"/>
+      <c r="F170" s="5" t="inlineStr">
+        <is>
+          <t>Невизначеність США-Іран обмежує зростання на Перській затоці Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G170" s="5" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -10113,7 +10789,11 @@
           <t>Єгипет підвищив ціни на газ для промисловості</t>
         </is>
       </c>
-      <c r="F171" s="5" t="inlineStr"/>
+      <c r="F171" s="5" t="inlineStr">
+        <is>
+          <t>Єгипет підвищив ціни на газ для промисловості Домен: енергетика Країна: Єгипет</t>
+        </is>
+      </c>
       <c r="G171" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -10171,7 +10851,11 @@
           <t>Продаж американського сланцевого оператора за 4+ млрд дол</t>
         </is>
       </c>
-      <c r="F172" s="5" t="inlineStr"/>
+      <c r="F172" s="5" t="inlineStr">
+        <is>
+          <t>Продаж американського сланцевого оператора за 4+ млрд дол Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G172" s="5" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -10229,7 +10913,11 @@
           <t>Японські власники танкерів отримують рекордні ціни</t>
         </is>
       </c>
-      <c r="F173" s="8" t="inlineStr"/>
+      <c r="F173" s="8" t="inlineStr">
+        <is>
+          <t>Японські власники танкерів отримують рекордні ціни Домен: логістика Країна: Японія</t>
+        </is>
+      </c>
       <c r="G173" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -10287,7 +10975,11 @@
           <t>Singapore Airlines затримує люкс-сидіння через ланцюг постачання</t>
         </is>
       </c>
-      <c r="F174" s="8" t="inlineStr"/>
+      <c r="F174" s="8" t="inlineStr">
+        <is>
+          <t>Singapore Airlines затримує люкс-сидіння через ланцюг постачання Домен: логістика Країна: Сінгапур</t>
+        </is>
+      </c>
       <c r="G174" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -10345,7 +11037,11 @@
           <t>Spirit Airlines припинила польоти</t>
         </is>
       </c>
-      <c r="F175" s="8" t="inlineStr"/>
+      <c r="F175" s="8" t="inlineStr">
+        <is>
+          <t>Spirit Airlines припинила польоти Домен: логістика Країна: США</t>
+        </is>
+      </c>
       <c r="G175" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -10399,7 +11095,11 @@
           <t>Трамп зустрічається з Лулою на економічні переговори</t>
         </is>
       </c>
-      <c r="F176" s="8" t="inlineStr"/>
+      <c r="F176" s="8" t="inlineStr">
+        <is>
+          <t>Трамп зустрічається з Лулою на економічні переговори Домен: геополітика Країна: Бразилія, США</t>
+        </is>
+      </c>
       <c r="G176" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -10453,7 +11153,11 @@
           <t>Крихке перемир'я в Перській затоці стабілізує золото</t>
         </is>
       </c>
-      <c r="F177" s="8" t="inlineStr"/>
+      <c r="F177" s="8" t="inlineStr">
+        <is>
+          <t>Крихке перемир'я в Перській затоці стабілізує золото Домен: геополітика Країна: Перська затока</t>
+        </is>
+      </c>
       <c r="G177" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -10511,7 +11215,11 @@
           <t>Грецькі судновласники замовляють нові судна на $10 млрд</t>
         </is>
       </c>
-      <c r="F178" s="8" t="inlineStr"/>
+      <c r="F178" s="8" t="inlineStr">
+        <is>
+          <t>Грецькі судновласники замовляють нові судна на $10 млрд Домен: логістика Країна: Греція</t>
+        </is>
+      </c>
       <c r="G178" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -10565,7 +11273,11 @@
           <t>ЄС виключив індійські верфі з реєстру переробки суден</t>
         </is>
       </c>
-      <c r="F179" s="8" t="inlineStr"/>
+      <c r="F179" s="8" t="inlineStr">
+        <is>
+          <t>ЄС виключив індійські верфі з реєстру переробки суден Домен: логістика Країна: Індія</t>
+        </is>
+      </c>
       <c r="G179" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -10619,7 +11331,11 @@
           <t>Запаси сирої нафти в США впали на 8,1 млн барелів</t>
         </is>
       </c>
-      <c r="F180" s="8" t="inlineStr"/>
+      <c r="F180" s="8" t="inlineStr">
+        <is>
+          <t>Запаси сирої нафти в США впали на 8,1 млн барелів Домен: ціни_сировини Країна: США</t>
+        </is>
+      </c>
       <c r="G180" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -10677,7 +11393,11 @@
           <t>Дохідність облігацій США досягла 5%</t>
         </is>
       </c>
-      <c r="F181" s="8" t="inlineStr"/>
+      <c r="F181" s="8" t="inlineStr">
+        <is>
+          <t>Дохідність облігацій США досягла 5% Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G181" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -10731,7 +11451,11 @@
           <t>Експерт попереджає про фіскальні ризики для долара США</t>
         </is>
       </c>
-      <c r="F182" s="8" t="inlineStr"/>
+      <c r="F182" s="8" t="inlineStr">
+        <is>
+          <t>Експерт попереджає про фіскальні ризики для долара США Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G182" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -10785,7 +11509,11 @@
           <t>Бразилія наближається до китайської квоти на яловичину</t>
         </is>
       </c>
-      <c r="F183" s="8" t="inlineStr"/>
+      <c r="F183" s="8" t="inlineStr">
+        <is>
+          <t>Бразилія наближається до китайської квоти на яловичину Домен: ціни_сировини Країна: Бразилія, Китай</t>
+        </is>
+      </c>
       <c r="G183" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -10843,7 +11571,11 @@
           <t>Угода про економію $64,3 млрд на цінах ліків за 10 років</t>
         </is>
       </c>
-      <c r="F184" s="8" t="inlineStr"/>
+      <c r="F184" s="8" t="inlineStr">
+        <is>
+          <t>Угода про економію $64,3 млрд на цінах ліків за 10 років Домен: ціни_сировини Країна: США</t>
+        </is>
+      </c>
       <c r="G184" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -10901,7 +11633,11 @@
           <t>G7 створює постійний орган для контролю критичних мінералів</t>
         </is>
       </c>
-      <c r="F185" s="8" t="inlineStr"/>
+      <c r="F185" s="8" t="inlineStr">
+        <is>
+          <t>G7 створює постійний орган для контролю критичних мінералів Домен: санкції_торгівля Країна: G7</t>
+        </is>
+      </c>
       <c r="G185" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -10959,7 +11695,11 @@
           <t>E-commerce експорт з Китаю впав на 6% у березні</t>
         </is>
       </c>
-      <c r="F186" s="8" t="inlineStr"/>
+      <c r="F186" s="8" t="inlineStr">
+        <is>
+          <t>E-commerce експорт з Китаю впав на 6% у березні Домен: логістика Країна: Китай</t>
+        </is>
+      </c>
       <c r="G186" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -11017,7 +11757,11 @@
           <t>Suzano отримує схвалення ЄС на угоду з Kimberly-Clark</t>
         </is>
       </c>
-      <c r="F187" s="8" t="inlineStr"/>
+      <c r="F187" s="8" t="inlineStr">
+        <is>
+          <t>Suzano отримує схвалення ЄС на угоду з Kimberly-Clark Домен: санкції_торгівля Країна: Бразилія, ЄС</t>
+        </is>
+      </c>
       <c r="G187" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -11075,7 +11819,11 @@
           <t>8 млн бразильських фірм не сплачують борги</t>
         </is>
       </c>
-      <c r="F188" s="8" t="inlineStr"/>
+      <c r="F188" s="8" t="inlineStr">
+        <is>
+          <t>8 млн бразильських фірм не сплачують борги Домен: валюта_фінанси Країна: Бразилія</t>
+        </is>
+      </c>
       <c r="G188" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -11129,7 +11877,11 @@
           <t>Російський суд конфіскує агроімперію олігарха</t>
         </is>
       </c>
-      <c r="F189" s="8" t="inlineStr"/>
+      <c r="F189" s="8" t="inlineStr">
+        <is>
+          <t>Російський суд конфіскує агроімперію олігарха Домен: геополітика Країна: Росія</t>
+        </is>
+      </c>
       <c r="G189" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -11187,7 +11939,11 @@
           <t>Зростання сектору послуг США сповільнилось на 3 роки</t>
         </is>
       </c>
-      <c r="F190" s="8" t="inlineStr"/>
+      <c r="F190" s="8" t="inlineStr">
+        <is>
+          <t>Зростання сектору послуг США сповільнилось на 3 роки Домен: геополітика Країна: США</t>
+        </is>
+      </c>
       <c r="G190" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -11241,7 +11997,11 @@
           <t>США пропонують пакт з електронної комерції на тлі дедлоку ВТО</t>
         </is>
       </c>
-      <c r="F191" s="8" t="inlineStr"/>
+      <c r="F191" s="8" t="inlineStr">
+        <is>
+          <t>США пропонують пакт з електронної комерції на тлі дедлоку ВТО Домен: санкції_торгівля Країна: США</t>
+        </is>
+      </c>
       <c r="G191" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -11295,7 +12055,11 @@
           <t>Chevron розширює газовидобуток у Середземномор'ї</t>
         </is>
       </c>
-      <c r="F192" s="8" t="inlineStr"/>
+      <c r="F192" s="8" t="inlineStr">
+        <is>
+          <t>Chevron розширює газовидобуток у Середземномор'ї Домен: ціни_сировини Країна: Мальта</t>
+        </is>
+      </c>
       <c r="G192" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -11353,7 +12117,11 @@
           <t>Cummins підвищує прогноз доходів через попит на генератори</t>
         </is>
       </c>
-      <c r="F193" s="8" t="inlineStr"/>
+      <c r="F193" s="8" t="inlineStr">
+        <is>
+          <t>Cummins підвищує прогноз доходів через попит на генератори Домен: ціни_сировини Країна: США</t>
+        </is>
+      </c>
       <c r="G193" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -11411,7 +12179,11 @@
           <t>Трейдери нафти навігують конфлікт з Іраном</t>
         </is>
       </c>
-      <c r="F194" s="8" t="inlineStr"/>
+      <c r="F194" s="8" t="inlineStr">
+        <is>
+          <t>Трейдери нафти навігують конфлікт з Іраном Домен: ціни_сировини Країна: Іран</t>
+        </is>
+      </c>
       <c r="G194" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -11469,7 +12241,11 @@
           <t>ADNOC розширює видобуток нафти та газу після виходу з ОПЕК</t>
         </is>
       </c>
-      <c r="F195" s="8" t="inlineStr"/>
+      <c r="F195" s="8" t="inlineStr">
+        <is>
+          <t>ADNOC розширює видобуток нафти та газу після виходу з ОПЕК Домен: ціни_сировини Країна: ОАЕ</t>
+        </is>
+      </c>
       <c r="G195" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -11527,7 +12303,11 @@
           <t>Норвегія пропонує до 70 нових дозволів на видобуток нафти та газу</t>
         </is>
       </c>
-      <c r="F196" s="8" t="inlineStr"/>
+      <c r="F196" s="8" t="inlineStr">
+        <is>
+          <t>Норвегія пропонує до 70 нових дозволів на видобуток нафти та газу Домен: ціни_сировини Країна: Норвегія</t>
+        </is>
+      </c>
       <c r="G196" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -11585,7 +12365,11 @@
           <t>Трубопровід Канада-США близький до цільового обсягу</t>
         </is>
       </c>
-      <c r="F197" s="8" t="inlineStr"/>
+      <c r="F197" s="8" t="inlineStr">
+        <is>
+          <t>Трубопровід Канада-США близький до цільового обсягу Домен: логістика Країна: Канада, США</t>
+        </is>
+      </c>
       <c r="G197" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -11643,7 +12427,11 @@
           <t>Бельгійський сектор комбікорму впевнений попри виклики</t>
         </is>
       </c>
-      <c r="F198" s="8" t="inlineStr"/>
+      <c r="F198" s="8" t="inlineStr">
+        <is>
+          <t>Бельгійський сектор комбікорму впевнений попри виклики Домен: ціни_сировини Країна: Бельгія</t>
+        </is>
+      </c>
       <c r="G198" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -11701,7 +12489,11 @@
           <t>INEOS та Shell досліджують нові можливості в Мексиканській затоці</t>
         </is>
       </c>
-      <c r="F199" s="8" t="inlineStr"/>
+      <c r="F199" s="8" t="inlineStr">
+        <is>
+          <t>INEOS та Shell досліджують нові можливості в Мексиканській затоці Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G199" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -11759,7 +12551,11 @@
           <t>Завершення Third Track поліпшує залізничну логістику</t>
         </is>
       </c>
-      <c r="F200" s="8" t="inlineStr"/>
+      <c r="F200" s="8" t="inlineStr">
+        <is>
+          <t>Завершення Third Track поліпшує залізничну логістику Домен: логістика Країна: Нідерланди, Німеччина</t>
+        </is>
+      </c>
       <c r="G200" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -11813,7 +12609,11 @@
           <t>Hugo Boss перевищив прибутки попри напруженість з Іраном</t>
         </is>
       </c>
-      <c r="F201" s="8" t="inlineStr"/>
+      <c r="F201" s="8" t="inlineStr">
+        <is>
+          <t>Hugo Boss перевищив прибутки попри напруженість з Іраном Домен: геополітика Країна: Іран, США</t>
+        </is>
+      </c>
       <c r="G201" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -11867,7 +12667,11 @@
           <t>Пакистан має достатні запаси сечовини на сезон</t>
         </is>
       </c>
-      <c r="F202" s="8" t="inlineStr"/>
+      <c r="F202" s="8" t="inlineStr">
+        <is>
+          <t>Пакистан має достатні запаси сечовини на сезон Домен: ціни_сировини Країна: Пакистан</t>
+        </is>
+      </c>
       <c r="G202" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -11925,7 +12729,11 @@
           <t>РБА Австралії припиняє цикл підвищення ставок</t>
         </is>
       </c>
-      <c r="F203" s="8" t="inlineStr"/>
+      <c r="F203" s="8" t="inlineStr">
+        <is>
+          <t>РБА Австралії припиняє цикл підвищення ставок Домен: валюта_фінанси Країна: Австралія</t>
+        </is>
+      </c>
       <c r="G203" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -11979,7 +12787,11 @@
           <t>SEMI прогнозує стійкий попит на чіпи попри ризики</t>
         </is>
       </c>
-      <c r="F204" s="8" t="inlineStr"/>
+      <c r="F204" s="8" t="inlineStr">
+        <is>
+          <t>SEMI прогнозує стійкий попит на чіпи попри ризики Домен: санкції_торгівля Країна: глобально</t>
+        </is>
+      </c>
       <c r="G204" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -12037,7 +12849,11 @@
           <t>Індійські дилери готуються до наслідків конфлікту</t>
         </is>
       </c>
-      <c r="F205" s="8" t="inlineStr"/>
+      <c r="F205" s="8" t="inlineStr">
+        <is>
+          <t>Індійські дилери готуються до наслідків конфлікту Домен: геополітика Країна: Індія</t>
+        </is>
+      </c>
       <c r="G205" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -12091,7 +12907,11 @@
           <t>Злиття гірничих компаній впливає на ціни золота</t>
         </is>
       </c>
-      <c r="F206" s="8" t="inlineStr"/>
+      <c r="F206" s="8" t="inlineStr">
+        <is>
+          <t>Злиття гірничих компаній впливає на ціни золота Домен: ціни_сировини</t>
+        </is>
+      </c>
       <c r="G206" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -12145,7 +12965,11 @@
           <t>Золото зростає на фоні близькосхідних ризиків</t>
         </is>
       </c>
-      <c r="F207" s="8" t="inlineStr"/>
+      <c r="F207" s="8" t="inlineStr">
+        <is>
+          <t>Золото зростає на фоні близькосхідних ризиків Домен: ціни_сировини</t>
+        </is>
+      </c>
       <c r="G207" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -12199,7 +13023,11 @@
           <t>ЄС рекомендує не використовувати Huawei і ZTE в інфраструктурі</t>
         </is>
       </c>
-      <c r="F208" s="8" t="inlineStr"/>
+      <c r="F208" s="8" t="inlineStr">
+        <is>
+          <t>ЄС рекомендує не використовувати Huawei і ZTE в інфраструктурі Домен: санкції_торгівля Країна: ЄС</t>
+        </is>
+      </c>
       <c r="G208" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -12257,7 +13085,11 @@
           <t>Diamondback збільшує видобуток нафти на хвилі зростання цін</t>
         </is>
       </c>
-      <c r="F209" s="8" t="inlineStr"/>
+      <c r="F209" s="8" t="inlineStr">
+        <is>
+          <t>Diamondback збільшує видобуток нафти на хвилі зростання цін Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G209" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -12311,7 +13143,11 @@
           <t>Канадські нафтові фірми борються з податком на вуглець</t>
         </is>
       </c>
-      <c r="F210" s="8" t="inlineStr"/>
+      <c r="F210" s="8" t="inlineStr">
+        <is>
+          <t>Канадські нафтові фірми борються з податком на вуглець Домен: енергетика Країна: Канада</t>
+        </is>
+      </c>
       <c r="G210" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -12369,7 +13205,11 @@
           <t>Італія посилює енергетичні зв'язки з Азербайджаном</t>
         </is>
       </c>
-      <c r="F211" s="8" t="inlineStr"/>
+      <c r="F211" s="8" t="inlineStr">
+        <is>
+          <t>Італія посилює енергетичні зв'язки з Азербайджаном Домен: енергетика Країна: Італія, Азербайджан</t>
+        </is>
+      </c>
       <c r="G211" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -12427,7 +13267,11 @@
           <t>Amazon переформатує логістику, UPS/FedEx падають</t>
         </is>
       </c>
-      <c r="F212" s="8" t="inlineStr"/>
+      <c r="F212" s="8" t="inlineStr">
+        <is>
+          <t>Amazon переформатує логістику, UPS/FedEx падають Домен: логістика</t>
+        </is>
+      </c>
       <c r="G212" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -12477,7 +13321,11 @@
           <t>Гайана в суді: Венесуела загрожує нафтовому регіону</t>
         </is>
       </c>
-      <c r="F213" s="8" t="inlineStr"/>
+      <c r="F213" s="8" t="inlineStr">
+        <is>
+          <t>Гайана в суді: Венесуела загрожує нафтовому регіону Домен: геополітика Країна: Гайана, Венесуела</t>
+        </is>
+      </c>
       <c r="G213" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -12535,7 +13383,11 @@
           <t>DOJ планує врегулювати справу AgriStats щодо цін на сільгосп</t>
         </is>
       </c>
-      <c r="F214" s="8" t="inlineStr"/>
+      <c r="F214" s="8" t="inlineStr">
+        <is>
+          <t>DOJ планує врегулювати справу AgriStats щодо цін на сільгосп Домен: санкції_торгівля Країна: США</t>
+        </is>
+      </c>
       <c r="G214" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -12589,7 +13441,11 @@
           <t>Європейські акції падають через ситуацію на Близькому Сході</t>
         </is>
       </c>
-      <c r="F215" s="8" t="inlineStr"/>
+      <c r="F215" s="8" t="inlineStr">
+        <is>
+          <t>Європейські акції падають через ситуацію на Близькому Сході Домен: геополітика Країна: Європа, Близький Схід</t>
+        </is>
+      </c>
       <c r="G215" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -12643,7 +13499,11 @@
           <t>Інтенсивна спека в Індії підняла видобуток електроенергії на 2-річний максимум</t>
         </is>
       </c>
-      <c r="F216" s="8" t="inlineStr"/>
+      <c r="F216" s="8" t="inlineStr">
+        <is>
+          <t>Інтенсивна спека в Індії підняла видобуток електроенергії на 2-річний максимум Домен: енергетика Країна: Індія</t>
+        </is>
+      </c>
       <c r="G216" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -12701,7 +13561,11 @@
           <t>Висока ціна нафти не врятує російське економічне зростання</t>
         </is>
       </c>
-      <c r="F217" s="8" t="inlineStr"/>
+      <c r="F217" s="8" t="inlineStr">
+        <is>
+          <t>Висока ціна нафти не врятує російське економічне зростання Домен: ціни_сировини Країна: Росія</t>
+        </is>
+      </c>
       <c r="G217" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -12759,7 +13623,11 @@
           <t>Reliance скорочує експорт алкілатів, збільшує LPG</t>
         </is>
       </c>
-      <c r="F218" s="8" t="inlineStr"/>
+      <c r="F218" s="8" t="inlineStr">
+        <is>
+          <t>Reliance скорочує експорт алкілатів, збільшує LPG Домен: енергетика Країна: Індія</t>
+        </is>
+      </c>
       <c r="G218" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -12817,7 +13685,11 @@
           <t>Saudi Aramco утримує LPG, Sonatrach знижує на 2-18%</t>
         </is>
       </c>
-      <c r="F219" s="8" t="inlineStr"/>
+      <c r="F219" s="8" t="inlineStr">
+        <is>
+          <t>Saudi Aramco утримує LPG, Sonatrach знижує на 2-18% Домен: ціни_сировини Країна: Саудівська Аравія, Алжир</t>
+        </is>
+      </c>
       <c r="G219" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -12875,7 +13747,11 @@
           <t>ОАЕ наполягає на необмеженому видобутку</t>
         </is>
       </c>
-      <c r="F220" s="8" t="inlineStr"/>
+      <c r="F220" s="8" t="inlineStr">
+        <is>
+          <t>ОАЕ наполягає на необмеженому видобутку Домен: енергетика Країна: ОАЕ</t>
+        </is>
+      </c>
       <c r="G220" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -12933,7 +13809,11 @@
           <t>Китайський юань може зміцнитися проти долара</t>
         </is>
       </c>
-      <c r="F221" s="8" t="inlineStr"/>
+      <c r="F221" s="8" t="inlineStr">
+        <is>
+          <t>Китайський юань може зміцнитися проти долара Домен: валюта_фінанси Країна: Китай</t>
+        </is>
+      </c>
       <c r="G221" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -12987,7 +13867,11 @@
           <t>Настрої інвесторів в єврозоні дещо поліпшилися</t>
         </is>
       </c>
-      <c r="F222" s="8" t="inlineStr"/>
+      <c r="F222" s="8" t="inlineStr">
+        <is>
+          <t>Настрої інвесторів в єврозоні дещо поліпшилися Домен: валюта_фінанси Країна: Єврозона</t>
+        </is>
+      </c>
       <c r="G222" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -13041,7 +13925,11 @@
           <t>Європейські заводи закуповували сировину, але оптимізм впав</t>
         </is>
       </c>
-      <c r="F223" s="8" t="inlineStr"/>
+      <c r="F223" s="8" t="inlineStr">
+        <is>
+          <t>Європейські заводи закуповували сировину, але оптимізм впав Домен: ціни_сировини Країна: Єврозона</t>
+        </is>
+      </c>
       <c r="G223" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -13099,7 +13987,11 @@
           <t>США евакуювали екіпаж захопленого іранського судна</t>
         </is>
       </c>
-      <c r="F224" s="8" t="inlineStr"/>
+      <c r="F224" s="8" t="inlineStr">
+        <is>
+          <t>США евакуювали екіпаж захопленого іранського судна Домен: геополітика Країна: Іран</t>
+        </is>
+      </c>
       <c r="G224" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -13153,7 +14045,11 @@
           <t>Індія відновила експорт пшениці після 4 років</t>
         </is>
       </c>
-      <c r="F225" s="8" t="inlineStr"/>
+      <c r="F225" s="8" t="inlineStr">
+        <is>
+          <t>Індія відновила експорт пшениці після 4 років Домен: ціни_сировини Країна: Індія</t>
+        </is>
+      </c>
       <c r="G225" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -13211,7 +14107,11 @@
           <t>Сервісна стратегія критична для успіху автоматизації інкубаторів</t>
         </is>
       </c>
-      <c r="F226" s="8" t="inlineStr"/>
+      <c r="F226" s="8" t="inlineStr">
+        <is>
+          <t>Сервісна стратегія критична для успіху автоматизації інкубаторів Домен: логістика Країна: світ</t>
+        </is>
+      </c>
       <c r="G226" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -13269,7 +14169,11 @@
           <t>Британське птахівництво під тиском через викиди аміаку</t>
         </is>
       </c>
-      <c r="F227" s="8" t="inlineStr"/>
+      <c r="F227" s="8" t="inlineStr">
+        <is>
+          <t>Британське птахівництво під тиском через викиди аміаку Домен: санкції_торгівля Країна: Великобританія</t>
+        </is>
+      </c>
       <c r="G227" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -13327,7 +14231,11 @@
           <t>Індійські акції зростають на тлі зниження цін на нафту</t>
         </is>
       </c>
-      <c r="F228" s="8" t="inlineStr"/>
+      <c r="F228" s="8" t="inlineStr">
+        <is>
+          <t>Індійські акції зростають на тлі зниження цін на нафту Домен: ціни_сировини Країна: Індія</t>
+        </is>
+      </c>
       <c r="G228" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -13385,7 +14293,11 @@
           <t>Австралійська рафінерія перезапускає виробництво в червні</t>
         </is>
       </c>
-      <c r="F229" s="8" t="inlineStr"/>
+      <c r="F229" s="8" t="inlineStr">
+        <is>
+          <t>Австралійська рафінерія перезапускає виробництво в червні Домен: енергетика Країна: Австралія</t>
+        </is>
+      </c>
       <c r="G229" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -13443,7 +14355,11 @@
           <t>ЕЦБ занепокоєна рецесією в Європі</t>
         </is>
       </c>
-      <c r="F230" s="8" t="inlineStr"/>
+      <c r="F230" s="8" t="inlineStr">
+        <is>
+          <t>ЕЦБ занепокоєна рецесією в Європі Домен: ціни_сировини Країна: ЄС</t>
+        </is>
+      </c>
       <c r="G230" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -13497,7 +14413,11 @@
           <t>Повені в Кенії, 18 загиблих</t>
         </is>
       </c>
-      <c r="F231" s="8" t="inlineStr"/>
+      <c r="F231" s="8" t="inlineStr">
+        <is>
+          <t>Повені в Кенії, 18 загиблих Домен: погода_клімат Країна: Кенія</t>
+        </is>
+      </c>
       <c r="G231" s="8" t="inlineStr">
         <is>
           <t>погода_клімат</t>
@@ -13551,7 +14471,11 @@
           <t>Шведський берегова охорона затримала танкер у Балтиці</t>
         </is>
       </c>
-      <c r="F232" s="8" t="inlineStr"/>
+      <c r="F232" s="8" t="inlineStr">
+        <is>
+          <t>Шведський берегова охорона затримала танкер у Балтиці Домен: логістика Країна: Швеція</t>
+        </is>
+      </c>
       <c r="G232" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -13605,7 +14529,11 @@
           <t>Виборці судитимуть Трампа за економіку</t>
         </is>
       </c>
-      <c r="F233" s="8" t="inlineStr"/>
+      <c r="F233" s="8" t="inlineStr">
+        <is>
+          <t>Виборці судитимуть Трампа за економіку Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G233" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -13659,7 +14587,11 @@
           <t>Китай та Філіппіни обмінюються звинуваченнями у морі</t>
         </is>
       </c>
-      <c r="F234" s="8" t="inlineStr"/>
+      <c r="F234" s="8" t="inlineStr">
+        <is>
+          <t>Китай та Філіппіни обмінюються звинуваченнями у морі Домен: геополітика Країна: Китай</t>
+        </is>
+      </c>
       <c r="G234" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -13713,7 +14645,11 @@
           <t>Про-ЄС уряд Румунії впав після голосування про недовіру</t>
         </is>
       </c>
-      <c r="F235" s="8" t="inlineStr"/>
+      <c r="F235" s="8" t="inlineStr">
+        <is>
+          <t>Про-ЄС уряд Румунії впав після голосування про недовіру Домен: геополітика Країна: Румунія</t>
+        </is>
+      </c>
       <c r="G235" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -13767,7 +14703,11 @@
           <t>Китайські послуги зростають попри цінові шоки</t>
         </is>
       </c>
-      <c r="F236" s="8" t="inlineStr"/>
+      <c r="F236" s="8" t="inlineStr">
+        <is>
+          <t>Китайські послуги зростають попри цінові шоки Домен: ціни_сировини Країна: Китай</t>
+        </is>
+      </c>
       <c r="G236" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -13821,7 +14761,11 @@
           <t>Fitch підвищує рейтинг Аргентини на B- через реформи</t>
         </is>
       </c>
-      <c r="F237" s="8" t="inlineStr"/>
+      <c r="F237" s="8" t="inlineStr">
+        <is>
+          <t>Fitch підвищує рейтинг Аргентини на B- через реформи Домен: валюта_фінанси Країна: Аргентина</t>
+        </is>
+      </c>
       <c r="G237" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -13875,7 +14819,11 @@
           <t>Лула піднімає тему організованої злочинності на зустрічі з Трампом</t>
         </is>
       </c>
-      <c r="F238" s="8" t="inlineStr"/>
+      <c r="F238" s="8" t="inlineStr">
+        <is>
+          <t>Лула піднімає тему організованої злочинності на зустрічі з Трампом Домен: геополітика Країна: Бразилія</t>
+        </is>
+      </c>
       <c r="G238" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -13929,7 +14877,11 @@
           <t>Перемога Моді стимулює індійські промислові акції</t>
         </is>
       </c>
-      <c r="F239" s="8" t="inlineStr"/>
+      <c r="F239" s="8" t="inlineStr">
+        <is>
+          <t>Перемога Моді стимулює індійські промислові акції Домен: геополітика Країна: Індія</t>
+        </is>
+      </c>
       <c r="G239" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -13983,7 +14935,11 @@
           <t>Азійські акції слідують за США на оптимізмі перемир'я</t>
         </is>
       </c>
-      <c r="F240" s="8" t="inlineStr"/>
+      <c r="F240" s="8" t="inlineStr">
+        <is>
+          <t>Азійські акції слідують за США на оптимізмі перемир'я Домен: геополітика Країна: Азія</t>
+        </is>
+      </c>
       <c r="G240" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -14037,7 +14993,11 @@
           <t>Нафта падає після заяви США про завершення наступу на Іран</t>
         </is>
       </c>
-      <c r="F241" s="8" t="inlineStr"/>
+      <c r="F241" s="8" t="inlineStr">
+        <is>
+          <t>Нафта падає після заяви США про завершення наступу на Іран Домен: енергетика Країна: США</t>
+        </is>
+      </c>
       <c r="G241" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -14091,7 +15051,11 @@
           <t>Судно перенаправлено до порту Гвадар через регіональну ситуацію</t>
         </is>
       </c>
-      <c r="F242" s="8" t="inlineStr"/>
+      <c r="F242" s="8" t="inlineStr">
+        <is>
+          <t>Судно перенаправлено до порту Гвадар через регіональну ситуацію Домен: логістика Країна: Пакистан</t>
+        </is>
+      </c>
       <c r="G242" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -14149,7 +15113,11 @@
           <t>AI трансформуватиме закупівлі до 2030 року</t>
         </is>
       </c>
-      <c r="F243" s="8" t="inlineStr"/>
+      <c r="F243" s="8" t="inlineStr">
+        <is>
+          <t>AI трансформуватиме закупівлі до 2030 року</t>
+        </is>
+      </c>
       <c r="G243" s="8" t="inlineStr">
         <is>
           <t>не_релевантно</t>
@@ -14199,7 +15167,11 @@
           <t>ВВП Гонконгу виріс на 5,9% у Q1 2026</t>
         </is>
       </c>
-      <c r="F244" s="8" t="inlineStr"/>
+      <c r="F244" s="8" t="inlineStr">
+        <is>
+          <t>ВВП Гонконгу виріс на 5,9% у Q1 2026 Домен: геополітика Країна: Гонконг</t>
+        </is>
+      </c>
       <c r="G244" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -14253,7 +15225,11 @@
           <t>Damen відкрив судноремонтну верф у Дакарі</t>
         </is>
       </c>
-      <c r="F245" s="8" t="inlineStr"/>
+      <c r="F245" s="8" t="inlineStr">
+        <is>
+          <t>Damen відкрив судноремонтну верф у Дакарі Домен: логістика Країна: Сенегал</t>
+        </is>
+      </c>
       <c r="G245" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -14307,7 +15283,11 @@
           <t>Трамп і Сі Цзіньпін обговорюватимуть Тайвань</t>
         </is>
       </c>
-      <c r="F246" s="8" t="inlineStr"/>
+      <c r="F246" s="8" t="inlineStr">
+        <is>
+          <t>Трамп і Сі Цзіньпін обговорюватимуть Тайвань Домен: геополітика Країна: США, Китай</t>
+        </is>
+      </c>
       <c r="G246" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -14361,7 +15341,11 @@
           <t>Мексика планує інвестувати $12 млрд в інфраструктуру</t>
         </is>
       </c>
-      <c r="F247" s="8" t="inlineStr"/>
+      <c r="F247" s="8" t="inlineStr">
+        <is>
+          <t>Мексика планує інвестувати $12 млрд в інфраструктуру Домен: геополітика Країна: Мексика</t>
+        </is>
+      </c>
       <c r="G247" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -14415,7 +15399,11 @@
           <t>Судан відкликав посла з Ефіопії через атаки на Хартум</t>
         </is>
       </c>
-      <c r="F248" s="8" t="inlineStr"/>
+      <c r="F248" s="8" t="inlineStr">
+        <is>
+          <t>Судан відкликав посла з Ефіопії через атаки на Хартум Домен: геополітика Країна: Судан, Ефіопія</t>
+        </is>
+      </c>
       <c r="G248" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -14469,7 +15457,11 @@
           <t>Вакансії в США впали, найми зросли</t>
         </is>
       </c>
-      <c r="F249" s="8" t="inlineStr"/>
+      <c r="F249" s="8" t="inlineStr">
+        <is>
+          <t>Вакансії в США впали, найми зросли Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G249" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -14523,7 +15515,11 @@
           <t>Європа потребує більших банків для конкуренції з США та Китаєм</t>
         </is>
       </c>
-      <c r="F250" s="8" t="inlineStr"/>
+      <c r="F250" s="8" t="inlineStr">
+        <is>
+          <t>Європа потребує більших банків для конкуренції з США та Китаєм Домен: валюта_фінанси Країна: Європа</t>
+        </is>
+      </c>
       <c r="G250" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -14577,7 +15573,11 @@
           <t>CMA CGM розширює логістичну мережу в ОАЕ через AD Ports</t>
         </is>
       </c>
-      <c r="F251" s="8" t="inlineStr"/>
+      <c r="F251" s="8" t="inlineStr">
+        <is>
+          <t>CMA CGM розширює логістичну мережу в ОАЕ через AD Ports Домен: логістика Країна: ОАЕ</t>
+        </is>
+      </c>
       <c r="G251" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -14631,7 +15631,11 @@
           <t>IFEEDER додає звіти про вітаміни та амінокислоти для жуйних</t>
         </is>
       </c>
-      <c r="F252" s="8" t="inlineStr"/>
+      <c r="F252" s="8" t="inlineStr">
+        <is>
+          <t>IFEEDER додає звіти про вітаміни та амінокислоти для жуйних Домен: ціни_сировини</t>
+        </is>
+      </c>
       <c r="G252" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -14685,7 +15689,11 @@
           <t>Трубопровід США-Канада наближається до запуску</t>
         </is>
       </c>
-      <c r="F253" s="8" t="inlineStr"/>
+      <c r="F253" s="8" t="inlineStr">
+        <is>
+          <t>Трубопровід США-Канада наближається до запуску Домен: логістика Країна: США, Канада</t>
+        </is>
+      </c>
       <c r="G253" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -14743,7 +15751,11 @@
           <t>Морська стратегія Китаю дає зворотний ефект</t>
         </is>
       </c>
-      <c r="F254" s="8" t="inlineStr"/>
+      <c r="F254" s="8" t="inlineStr">
+        <is>
+          <t>Морська стратегія Китаю дає зворотний ефект Домен: геополітика Країна: Китай</t>
+        </is>
+      </c>
       <c r="G254" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -14797,7 +15809,11 @@
           <t>Cargill очолює Sea Cargo Charter для контролю викидів</t>
         </is>
       </c>
-      <c r="F255" s="8" t="inlineStr"/>
+      <c r="F255" s="8" t="inlineStr">
+        <is>
+          <t>Cargill очолює Sea Cargo Charter для контролю викидів Домен: логістика</t>
+        </is>
+      </c>
       <c r="G255" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -14847,7 +15863,11 @@
           <t>IPG Shipping розпочинає операції в Австралії</t>
         </is>
       </c>
-      <c r="F256" s="8" t="inlineStr"/>
+      <c r="F256" s="8" t="inlineStr">
+        <is>
+          <t>IPG Shipping розпочинає операції в Австралії Домен: логістика Країна: Австралія</t>
+        </is>
+      </c>
       <c r="G256" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -14905,7 +15925,11 @@
           <t>GlobalFoundries прогнозує зростання попиту на чипи</t>
         </is>
       </c>
-      <c r="F257" s="8" t="inlineStr"/>
+      <c r="F257" s="8" t="inlineStr">
+        <is>
+          <t>GlobalFoundries прогнозує зростання попиту на чипи Домен: ціни_сировини Країна: США</t>
+        </is>
+      </c>
       <c r="G257" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -14959,7 +15983,11 @@
           <t>Румунський уряд впав, під загрозою фіскальні реформи</t>
         </is>
       </c>
-      <c r="F258" s="8" t="inlineStr"/>
+      <c r="F258" s="8" t="inlineStr">
+        <is>
+          <t>Румунський уряд впав, під загрозою фіскальні реформи Домен: санкції_торгівля Країна: Румунія</t>
+        </is>
+      </c>
       <c r="G258" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -15013,7 +16041,11 @@
           <t>ВВП Індонезії зростає на 5.6% попри конфлікт</t>
         </is>
       </c>
-      <c r="F259" s="8" t="inlineStr"/>
+      <c r="F259" s="8" t="inlineStr">
+        <is>
+          <t>ВВП Індонезії зростає на 5.6% попри конфлікт Домен: ціни_сировини Країна: Індонезія</t>
+        </is>
+      </c>
       <c r="G259" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -15067,7 +16099,11 @@
           <t>Соєвий шрот тестує ключовий рівень підтримки</t>
         </is>
       </c>
-      <c r="F260" s="8" t="inlineStr"/>
+      <c r="F260" s="8" t="inlineStr">
+        <is>
+          <t>Соєвий шрот тестує ключовий рівень підтримки Домен: ціни_сировини</t>
+        </is>
+      </c>
       <c r="G260" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -15121,7 +16157,11 @@
           <t>Норвегія приєднується до США для захисту ланцюгів AI</t>
         </is>
       </c>
-      <c r="F261" s="8" t="inlineStr"/>
+      <c r="F261" s="8" t="inlineStr">
+        <is>
+          <t>Норвегія приєднується до США для захисту ланцюгів AI Домен: санкції_торгівля Країна: Норвегія, США</t>
+        </is>
+      </c>
       <c r="G261" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -15175,7 +16215,11 @@
           <t>Білі несучки набирають популярність у Великобританії</t>
         </is>
       </c>
-      <c r="F262" s="8" t="inlineStr"/>
+      <c r="F262" s="8" t="inlineStr">
+        <is>
+          <t>Білі несучки набирають популярність у Великобританії Країна: Великобританія</t>
+        </is>
+      </c>
       <c r="G262" s="8" t="inlineStr">
         <is>
           <t>не_релевантно</t>
@@ -15229,7 +16273,11 @@
           <t>Таїланд розриває 25-річну угоду з Камбоджею про енергію</t>
         </is>
       </c>
-      <c r="F263" s="8" t="inlineStr"/>
+      <c r="F263" s="8" t="inlineStr">
+        <is>
+          <t>Таїланд розриває 25-річну угоду з Камбоджею про енергію Домен: геополітика Країна: Таїланд, Камбоджа</t>
+        </is>
+      </c>
       <c r="G263" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -15287,7 +16335,11 @@
           <t>Річка в Індонезії вийшла з берегів через сильні дощі</t>
         </is>
       </c>
-      <c r="F264" s="8" t="inlineStr"/>
+      <c r="F264" s="8" t="inlineStr">
+        <is>
+          <t>Річка в Індонезії вийшла з берегів через сильні дощі Домен: погода_клімат Країна: Індонезія</t>
+        </is>
+      </c>
       <c r="G264" s="8" t="inlineStr">
         <is>
           <t>погода_клімат</t>
@@ -15341,7 +16393,11 @@
           <t>Готівкові зняття в Індії зросли на 12% на початку квітня</t>
         </is>
       </c>
-      <c r="F265" s="8" t="inlineStr"/>
+      <c r="F265" s="8" t="inlineStr">
+        <is>
+          <t>Готівкові зняття в Індії зросли на 12% на початку квітня Домен: валюта_фінанси Країна: Індія</t>
+        </is>
+      </c>
       <c r="G265" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -15395,7 +16451,11 @@
           <t>Китайські автовиробці прагнуть глобального зростання</t>
         </is>
       </c>
-      <c r="F266" s="8" t="inlineStr"/>
+      <c r="F266" s="8" t="inlineStr">
+        <is>
+          <t>Китайські автовиробці прагнуть глобального зростання Домен: геополітика Країна: Китай</t>
+        </is>
+      </c>
       <c r="G266" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -15449,7 +16509,11 @@
           <t>Індонезія показує найшвидше зростання за три роки</t>
         </is>
       </c>
-      <c r="F267" s="8" t="inlineStr"/>
+      <c r="F267" s="8" t="inlineStr">
+        <is>
+          <t>Індонезія показує найшвидше зростання за три роки Домен: геополітика Країна: Індонезія</t>
+        </is>
+      </c>
       <c r="G267" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -15503,7 +16567,11 @@
           <t>Президент Тайваню критикує спроби Китаю блокувати візити</t>
         </is>
       </c>
-      <c r="F268" s="8" t="inlineStr"/>
+      <c r="F268" s="8" t="inlineStr">
+        <is>
+          <t>Президент Тайваню критикує спроби Китаю блокувати візити Домен: геополітика Країна: Тайвань, Китай</t>
+        </is>
+      </c>
       <c r="G268" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -15557,7 +16625,11 @@
           <t>Меркель розробляє стратегію для Трампа</t>
         </is>
       </c>
-      <c r="F269" s="8" t="inlineStr"/>
+      <c r="F269" s="8" t="inlineStr">
+        <is>
+          <t>Меркель розробляє стратегію для Трампа Домен: санкції_торгівля Країна: Німеччина, США</t>
+        </is>
+      </c>
       <c r="G269" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -15611,7 +16683,11 @@
           <t>Президент зупинив гірничий проект через протести</t>
         </is>
       </c>
-      <c r="F270" s="8" t="inlineStr"/>
+      <c r="F270" s="8" t="inlineStr">
+        <is>
+          <t>Президент зупинив гірничий проект через протести Домен: геополітика Країна: Домініканська Республіка</t>
+        </is>
+      </c>
       <c r="G270" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -15665,7 +16741,11 @@
           <t>S&amp;P 500 впав через конфлікт на Близькому Сході</t>
         </is>
       </c>
-      <c r="F271" s="8" t="inlineStr"/>
+      <c r="F271" s="8" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 впав через конфлікт на Близькому Сході Домен: геополітика Країна: США</t>
+        </is>
+      </c>
       <c r="G271" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -15719,7 +16799,11 @@
           <t>Бразилія відновлює програму допомоги споживачам</t>
         </is>
       </c>
-      <c r="F272" s="8" t="inlineStr"/>
+      <c r="F272" s="8" t="inlineStr">
+        <is>
+          <t>Бразилія відновлює програму допомоги споживачам Домен: валюта_фінанси Країна: Бразилія</t>
+        </is>
+      </c>
       <c r="G272" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -15773,7 +16857,11 @@
           <t>Казначейство США збільшує прогноз запозичень на Q2</t>
         </is>
       </c>
-      <c r="F273" s="8" t="inlineStr"/>
+      <c r="F273" s="8" t="inlineStr">
+        <is>
+          <t>Казначейство США збільшує прогноз запозичень на Q2 Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G273" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -15827,7 +16915,11 @@
           <t>Глобальні фінансові лідери обговорюють потоки капіталу та AI</t>
         </is>
       </c>
-      <c r="F274" s="8" t="inlineStr"/>
+      <c r="F274" s="8" t="inlineStr">
+        <is>
+          <t>Глобальні фінансові лідери обговорюють потоки капіталу та AI Домен: валюта_фінанси</t>
+        </is>
+      </c>
       <c r="G274" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -15877,7 +16969,11 @@
           <t>Гайана: інвестицій в енергетику недостатньо</t>
         </is>
       </c>
-      <c r="F275" s="8" t="inlineStr"/>
+      <c r="F275" s="8" t="inlineStr">
+        <is>
+          <t>Гайана: інвестицій в енергетику недостатньо Домен: енергетика Країна: Гайана</t>
+        </is>
+      </c>
       <c r="G275" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -15935,7 +17031,11 @@
           <t>ЄС дає промисловості більше вільних дозволів CO2</t>
         </is>
       </c>
-      <c r="F276" s="8" t="inlineStr"/>
+      <c r="F276" s="8" t="inlineStr">
+        <is>
+          <t>ЄС дає промисловості більше вільних дозволів CO2 Домен: митниця_регуляторика Країна: ЄС</t>
+        </is>
+      </c>
       <c r="G276" s="8" t="inlineStr">
         <is>
           <t>митниця_регуляторика</t>
@@ -15989,7 +17089,11 @@
           <t>Паніка та хаос в FDA під керівництвом Марті Макарі</t>
         </is>
       </c>
-      <c r="F277" s="8" t="inlineStr"/>
+      <c r="F277" s="8" t="inlineStr">
+        <is>
+          <t>Паніка та хаос в FDA під керівництвом Марті Макарі Домен: здоров'я_біобезпека Країна: США</t>
+        </is>
+      </c>
       <c r="G277" s="8" t="inlineStr">
         <is>
           <t>здоров'я_біобезпека</t>
@@ -16043,7 +17147,11 @@
           <t>Tyson Foods перевищив прибуток, але яловичина слабка</t>
         </is>
       </c>
-      <c r="F278" s="8" t="inlineStr"/>
+      <c r="F278" s="8" t="inlineStr">
+        <is>
+          <t>Tyson Foods перевищив прибуток, але яловичина слабка Домен: ціни_сировини Країна: США</t>
+        </is>
+      </c>
       <c r="G278" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -16101,7 +17209,11 @@
           <t>Мерц відзначає рік у посаді серед трансатлантичної кризи</t>
         </is>
       </c>
-      <c r="F279" s="8" t="inlineStr"/>
+      <c r="F279" s="8" t="inlineStr">
+        <is>
+          <t>Мерц відзначає рік у посаді серед трансатлантичної кризи Домен: санкції_торгівля Країна: Німеччина, США</t>
+        </is>
+      </c>
       <c r="G279" s="8" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -16155,7 +17267,11 @@
           <t>Oaktree Co-CEO називає ціноутворення на ринку дивним</t>
         </is>
       </c>
-      <c r="F280" s="8" t="inlineStr"/>
+      <c r="F280" s="8" t="inlineStr">
+        <is>
+          <t>Oaktree Co-CEO називає ціноутворення на ринку дивним Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G280" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -16209,7 +17325,11 @@
           <t>Російна нафта зросла до $95/барель у квітні</t>
         </is>
       </c>
-      <c r="F281" s="8" t="inlineStr"/>
+      <c r="F281" s="8" t="inlineStr">
+        <is>
+          <t>Російна нафта зросла до $95/барель у квітні Домен: геополітика Країна: Росія</t>
+        </is>
+      </c>
       <c r="G281" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -16267,7 +17387,11 @@
           <t>Замбія розділяє угоду про здоров'я та мінерали</t>
         </is>
       </c>
-      <c r="F282" s="8" t="inlineStr"/>
+      <c r="F282" s="8" t="inlineStr">
+        <is>
+          <t>Замбія розділяє угоду про здоров'я та мінерали Домен: геополітика Країна: Замбія</t>
+        </is>
+      </c>
       <c r="G282" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -16325,7 +17449,11 @@
           <t>Споживання LPG в Індії впало на 16.2% р/р</t>
         </is>
       </c>
-      <c r="F283" s="8" t="inlineStr"/>
+      <c r="F283" s="8" t="inlineStr">
+        <is>
+          <t>Споживання LPG в Індії впало на 16.2% р/р Домен: ціни_сировини Країна: Індія</t>
+        </is>
+      </c>
       <c r="G283" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -16383,7 +17511,11 @@
           <t>Японія та Австралія поглиблюють співпрацю на енергії</t>
         </is>
       </c>
-      <c r="F284" s="8" t="inlineStr"/>
+      <c r="F284" s="8" t="inlineStr">
+        <is>
+          <t>Японія та Австралія поглиблюють співпрацю на енергії Домен: геополітика Країна: Японія, Австралія</t>
+        </is>
+      </c>
       <c r="G284" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -16441,7 +17573,11 @@
           <t>Amazon відкриває логістичну мережу для інших компаній</t>
         </is>
       </c>
-      <c r="F285" s="8" t="inlineStr"/>
+      <c r="F285" s="8" t="inlineStr">
+        <is>
+          <t>Amazon відкриває логістичну мережу для інших компаній Домен: логістика Країна: США</t>
+        </is>
+      </c>
       <c r="G285" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -16495,7 +17631,11 @@
           <t>ЧД Карго перевезла більше вантажу у 2025 році</t>
         </is>
       </c>
-      <c r="F286" s="8" t="inlineStr"/>
+      <c r="F286" s="8" t="inlineStr">
+        <is>
+          <t>ЧД Карго перевезла більше вантажу у 2025 році Домен: логістика Країна: Чехія</t>
+        </is>
+      </c>
       <c r="G286" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -16549,7 +17689,11 @@
           <t>Казахські залізниці будують власний морський флот</t>
         </is>
       </c>
-      <c r="F287" s="8" t="inlineStr"/>
+      <c r="F287" s="8" t="inlineStr">
+        <is>
+          <t>Казахські залізниці будують власний морський флот Домен: логістика Країна: Казахстан</t>
+        </is>
+      </c>
       <c r="G287" s="8" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -16603,7 +17747,11 @@
           <t>Novonesis номінована на Sustainability Impact Award 2026</t>
         </is>
       </c>
-      <c r="F288" s="8" t="inlineStr"/>
+      <c r="F288" s="8" t="inlineStr">
+        <is>
+          <t>Novonesis номінована на Sustainability Impact Award 2026</t>
+        </is>
+      </c>
       <c r="G288" s="8" t="inlineStr">
         <is>
           <t>не_релевантно</t>
@@ -16657,7 +17805,11 @@
           <t>Японська єна зміцнюється через інтервенції на ринку</t>
         </is>
       </c>
-      <c r="F289" s="8" t="inlineStr"/>
+      <c r="F289" s="8" t="inlineStr">
+        <is>
+          <t>Японська єна зміцнюється через інтервенції на ринку Домен: валюта_фінанси Країна: Японія</t>
+        </is>
+      </c>
       <c r="G289" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -16711,7 +17863,11 @@
           <t>OPEC+ символічно збільшує видобуток нафти</t>
         </is>
       </c>
-      <c r="F290" s="8" t="inlineStr"/>
+      <c r="F290" s="8" t="inlineStr">
+        <is>
+          <t>OPEC+ символічно збільшує видобуток нафти Домен: ціни_сировини Країна: світ</t>
+        </is>
+      </c>
       <c r="G290" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -16769,7 +17925,11 @@
           <t>Південнокорейське виробництво на максимумі за 4 роки</t>
         </is>
       </c>
-      <c r="F291" s="8" t="inlineStr"/>
+      <c r="F291" s="8" t="inlineStr">
+        <is>
+          <t>Південнокорейське виробництво на максимумі за 4 роки Домен: ціни_сировини Країна: Південна Корея</t>
+        </is>
+      </c>
       <c r="G291" s="8" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -16823,7 +17983,11 @@
           <t>ФРС занепокоєна стресом у приватному кредиті</t>
         </is>
       </c>
-      <c r="F292" s="8" t="inlineStr"/>
+      <c r="F292" s="8" t="inlineStr">
+        <is>
+          <t>ФРС занепокоєна стресом у приватному кредиті Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G292" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -16877,7 +18041,11 @@
           <t>Азійські лідери готові протидіяти волатильності</t>
         </is>
       </c>
-      <c r="F293" s="8" t="inlineStr"/>
+      <c r="F293" s="8" t="inlineStr">
+        <is>
+          <t>Азійські лідери готові протидіяти волатильності Домен: валюта_фінанси Країна: Азія</t>
+        </is>
+      </c>
       <c r="G293" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -16931,7 +18099,11 @@
           <t>АБР запускає план $70 млрд для енергетики та цифри</t>
         </is>
       </c>
-      <c r="F294" s="8" t="inlineStr"/>
+      <c r="F294" s="8" t="inlineStr">
+        <is>
+          <t>АБР запускає план $70 млрд для енергетики та цифри Домен: енергетика Країна: Азія-Тихий океан</t>
+        </is>
+      </c>
       <c r="G294" s="8" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -16985,7 +18157,11 @@
           <t>Прем'єр Словаччини відвідає парад Перемоги в Москві</t>
         </is>
       </c>
-      <c r="F295" s="8" t="inlineStr"/>
+      <c r="F295" s="8" t="inlineStr">
+        <is>
+          <t>Прем'єр Словаччини відвідає парад Перемоги в Москві Домен: геополітика Країна: Словаччина</t>
+        </is>
+      </c>
       <c r="G295" s="8" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -17039,7 +18215,11 @@
           <t>Ріст цін на нафту підтримує американський фондовий ринок</t>
         </is>
       </c>
-      <c r="F296" s="8" t="inlineStr"/>
+      <c r="F296" s="8" t="inlineStr">
+        <is>
+          <t>Ріст цін на нафту підтримує американський фондовий ринок Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G296" s="8" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -17093,7 +18273,11 @@
           <t>Пізня снігова буря в Денвері може бути найбільшою сезону</t>
         </is>
       </c>
-      <c r="F297" s="11" t="inlineStr"/>
+      <c r="F297" s="11" t="inlineStr">
+        <is>
+          <t>Пізня снігова буря в Денвері може бути найбільшою сезону Домен: погода_клімат Країна: США</t>
+        </is>
+      </c>
       <c r="G297" s="11" t="inlineStr">
         <is>
           <t>погода_клімат</t>
@@ -17151,7 +18335,11 @@
           <t>IACS опублікував результати інспекції аварійного живлення</t>
         </is>
       </c>
-      <c r="F298" s="11" t="inlineStr"/>
+      <c r="F298" s="11" t="inlineStr">
+        <is>
+          <t>IACS опублікував результати інспекції аварійного живлення Домен: логістика</t>
+        </is>
+      </c>
       <c r="G298" s="11" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -17201,7 +18389,11 @@
           <t>Круїзний корабель з хантавірусом прямує на Канари</t>
         </is>
       </c>
-      <c r="F299" s="11" t="inlineStr"/>
+      <c r="F299" s="11" t="inlineStr">
+        <is>
+          <t>Круїзний корабель з хантавірусом прямує на Канари Домен: здоров'я_біобезпека Країна: Іспанія</t>
+        </is>
+      </c>
       <c r="G299" s="11" t="inlineStr">
         <is>
           <t>здоров'я_біобезпека</t>
@@ -17255,7 +18447,11 @@
           <t>Мамата Бандерджі втрачає владу в Західній Бенгалії</t>
         </is>
       </c>
-      <c r="F300" s="11" t="inlineStr"/>
+      <c r="F300" s="11" t="inlineStr">
+        <is>
+          <t>Мамата Бандерджі втрачає владу в Західній Бенгалії Домен: геополітика Країна: Індія</t>
+        </is>
+      </c>
       <c r="G300" s="11" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -17309,7 +18505,11 @@
           <t>Бомбардування Ізраїлем спричинило руйнування в Ліване</t>
         </is>
       </c>
-      <c r="F301" s="11" t="inlineStr"/>
+      <c r="F301" s="11" t="inlineStr">
+        <is>
+          <t>Бомбардування Ізраїлем спричинило руйнування в Ліване Домен: геополітика Країна: Ліван</t>
+        </is>
+      </c>
       <c r="G301" s="11" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -17363,7 +18563,11 @@
           <t>Оман запустив стандарти енергоефективності портів</t>
         </is>
       </c>
-      <c r="F302" s="11" t="inlineStr"/>
+      <c r="F302" s="11" t="inlineStr">
+        <is>
+          <t>Оман запустив стандарти енергоефективності портів Домен: енергетика Країна: Оман</t>
+        </is>
+      </c>
       <c r="G302" s="11" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -17417,7 +18621,11 @@
           <t>Препарати для схуднення збільшують попит на сироватку</t>
         </is>
       </c>
-      <c r="F303" s="11" t="inlineStr"/>
+      <c r="F303" s="11" t="inlineStr">
+        <is>
+          <t>Препарати для схуднення збільшують попит на сироватку Домен: ціни_сировини</t>
+        </is>
+      </c>
       <c r="G303" s="11" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -17471,7 +18679,11 @@
           <t>Exxon використовує AI для аналізу нафти Гайани</t>
         </is>
       </c>
-      <c r="F304" s="11" t="inlineStr"/>
+      <c r="F304" s="11" t="inlineStr">
+        <is>
+          <t>Exxon використовує AI для аналізу нафти Гайани Домен: ціни_сировини Країна: Гайана</t>
+        </is>
+      </c>
       <c r="G304" s="11" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -17529,7 +18741,11 @@
           <t>Засудження активістів Palestine Action за рейд на Elbit</t>
         </is>
       </c>
-      <c r="F305" s="11" t="inlineStr"/>
+      <c r="F305" s="11" t="inlineStr">
+        <is>
+          <t>Засудження активістів Palestine Action за рейд на Elbit Домен: геополітика Країна: Великобританія</t>
+        </is>
+      </c>
       <c r="G305" s="11" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -17583,7 +18799,11 @@
           <t>LATAM Cargo запускає рейси до Венесуели</t>
         </is>
       </c>
-      <c r="F306" s="11" t="inlineStr"/>
+      <c r="F306" s="11" t="inlineStr">
+        <is>
+          <t>LATAM Cargo запускає рейси до Венесуели Домен: санкції_торгівля Країна: Венесуела, США</t>
+        </is>
+      </c>
       <c r="G306" s="11" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -17637,7 +18857,11 @@
           <t>Novartis закриває німецький завод, скорочує 220 робіт</t>
         </is>
       </c>
-      <c r="F307" s="11" t="inlineStr"/>
+      <c r="F307" s="11" t="inlineStr">
+        <is>
+          <t>Novartis закриває німецький завод, скорочує 220 робіт Домен: геополітика Країна: Німеччина</t>
+        </is>
+      </c>
       <c r="G307" s="11" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -17695,7 +18919,11 @@
           <t>Що таке NACHO trade</t>
         </is>
       </c>
-      <c r="F308" s="11" t="inlineStr"/>
+      <c r="F308" s="11" t="inlineStr">
+        <is>
+          <t>Що таке NACHO trade Домен: санкції_торгівля</t>
+        </is>
+      </c>
       <c r="G308" s="11" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -17745,7 +18973,11 @@
           <t>Поштовий комітет ОАЕ полегшує доставку</t>
         </is>
       </c>
-      <c r="F309" s="11" t="inlineStr"/>
+      <c r="F309" s="11" t="inlineStr">
+        <is>
+          <t>Поштовий комітет ОАЕ полегшує доставку Домен: логістика Країна: ОАЕ</t>
+        </is>
+      </c>
       <c r="G309" s="11" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -17799,7 +19031,11 @@
           <t>Опозиційний альянс Нігерії розпадається перед виборами 2027</t>
         </is>
       </c>
-      <c r="F310" s="11" t="inlineStr"/>
+      <c r="F310" s="11" t="inlineStr">
+        <is>
+          <t>Опозиційний альянс Нігерії розпадається перед виборами 2027 Домен: геополітика Країна: Нігерія</t>
+        </is>
+      </c>
       <c r="G310" s="11" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -17853,7 +19089,11 @@
           <t>Банк Малійських островів шукає фінансування через конфлікт</t>
         </is>
       </c>
-      <c r="F311" s="11" t="inlineStr"/>
+      <c r="F311" s="11" t="inlineStr">
+        <is>
+          <t>Банк Малійських островів шукає фінансування через конфлікт Домен: геополітика Країна: Малійські острови</t>
+        </is>
+      </c>
       <c r="G311" s="11" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -17907,7 +19147,11 @@
           <t>Alphabet розміщує облігації в євро для фінансування AI</t>
         </is>
       </c>
-      <c r="F312" s="11" t="inlineStr"/>
+      <c r="F312" s="11" t="inlineStr">
+        <is>
+          <t>Alphabet розміщує облігації в євро для фінансування AI Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G312" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -17961,7 +19205,11 @@
           <t>Змішані результати Q1 для північноамериканських операторів</t>
         </is>
       </c>
-      <c r="F313" s="11" t="inlineStr"/>
+      <c r="F313" s="11" t="inlineStr">
+        <is>
+          <t>Змішані результати Q1 для північноамериканських операторів Домен: логістика Країна: Канада, США</t>
+        </is>
+      </c>
       <c r="G313" s="11" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -18015,7 +19263,11 @@
           <t>Вибух газу на шахті в Колумбії, 9 загиблих</t>
         </is>
       </c>
-      <c r="F314" s="11" t="inlineStr"/>
+      <c r="F314" s="11" t="inlineStr">
+        <is>
+          <t>Вибух газу на шахті в Колумбії, 9 загиблих Домен: здоров'я_біобезпека Країна: Колумбія</t>
+        </is>
+      </c>
       <c r="G314" s="11" t="inlineStr">
         <is>
           <t>здоров'я_біобезпека</t>
@@ -18073,7 +19325,11 @@
           <t>Вірменія проводить саміт ЄС, відходить від Росії</t>
         </is>
       </c>
-      <c r="F315" s="11" t="inlineStr"/>
+      <c r="F315" s="11" t="inlineStr">
+        <is>
+          <t>Вірменія проводить саміт ЄС, відходить від Росії Домен: геополітика Країна: Вірменія, ЄС</t>
+        </is>
+      </c>
       <c r="G315" s="11" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -18127,7 +19383,11 @@
           <t>Експорт кави з Уганди дещо зріс порівняно з минулим роком</t>
         </is>
       </c>
-      <c r="F316" s="11" t="inlineStr"/>
+      <c r="F316" s="11" t="inlineStr">
+        <is>
+          <t>Експорт кави з Уганди дещо зріс порівняно з минулим роком Домен: ціни_сировини Країна: Угорщина</t>
+        </is>
+      </c>
       <c r="G316" s="11" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -18185,7 +19445,11 @@
           <t>AB InBev повертається до зростання з кращими продажами пива</t>
         </is>
       </c>
-      <c r="F317" s="11" t="inlineStr"/>
+      <c r="F317" s="11" t="inlineStr">
+        <is>
+          <t>AB InBev повертається до зростання з кращими продажами пива Домен: ціни_сировини Країна: Бельгія</t>
+        </is>
+      </c>
       <c r="G317" s="11" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -18243,7 +19507,11 @@
           <t>США готують візові санкції проти Китаю</t>
         </is>
       </c>
-      <c r="F318" s="11" t="inlineStr"/>
+      <c r="F318" s="11" t="inlineStr">
+        <is>
+          <t>США готують візові санкції проти Китаю Домен: санкції_торгівля Країна: США, Китай</t>
+        </is>
+      </c>
       <c r="G318" s="11" t="inlineStr">
         <is>
           <t>санкції_торгівля</t>
@@ -18297,7 +19565,11 @@
           <t>Qantas оптимістичний щодо паливних поставок</t>
         </is>
       </c>
-      <c r="F319" s="11" t="inlineStr"/>
+      <c r="F319" s="11" t="inlineStr">
+        <is>
+          <t>Qantas оптимістичний щодо паливних поставок Домен: енергетика Країна: Австралія</t>
+        </is>
+      </c>
       <c r="G319" s="11" t="inlineStr">
         <is>
           <t>енергетика</t>
@@ -18355,7 +19627,11 @@
           <t>Європейські банки залишають ринки американцям</t>
         </is>
       </c>
-      <c r="F320" s="11" t="inlineStr"/>
+      <c r="F320" s="11" t="inlineStr">
+        <is>
+          <t>Європейські банки залишають ринки американцям Домен: валюта_фінанси Країна: Європа, США</t>
+        </is>
+      </c>
       <c r="G320" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -18409,7 +19685,11 @@
           <t>Літак United Airlines вдарив вантажівку при посадці</t>
         </is>
       </c>
-      <c r="F321" s="11" t="inlineStr"/>
+      <c r="F321" s="11" t="inlineStr">
+        <is>
+          <t>Літак United Airlines вдарив вантажівку при посадці Домен: логістика Країна: США</t>
+        </is>
+      </c>
       <c r="G321" s="11" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -18463,7 +19743,11 @@
           <t>Гуманоїдні роботи автоматизують сортування відходів</t>
         </is>
       </c>
-      <c r="F322" s="11" t="inlineStr"/>
+      <c r="F322" s="11" t="inlineStr">
+        <is>
+          <t>Гуманоїдні роботи автоматизують сортування відходів Домен: страйки_перебої Країна: Великобританія</t>
+        </is>
+      </c>
       <c r="G322" s="11" t="inlineStr">
         <is>
           <t>страйки_перебої</t>
@@ -18517,7 +19801,11 @@
           <t>Чилійське сміттєзвалище — найбільший емітент метану</t>
         </is>
       </c>
-      <c r="F323" s="11" t="inlineStr"/>
+      <c r="F323" s="11" t="inlineStr">
+        <is>
+          <t>Чилійське сміттєзвалище — найбільший емітент метану Домен: погода_клімат Країна: Чилі</t>
+        </is>
+      </c>
       <c r="G323" s="11" t="inlineStr">
         <is>
           <t>погода_клімат</t>
@@ -18571,7 +19859,11 @@
           <t>Southwest розглядає найм механіків для Boeing MAX 7</t>
         </is>
       </c>
-      <c r="F324" s="11" t="inlineStr"/>
+      <c r="F324" s="11" t="inlineStr">
+        <is>
+          <t>Southwest розглядає найм механіків для Boeing MAX 7 Домен: логістика Країна: США</t>
+        </is>
+      </c>
       <c r="G324" s="11" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -18625,7 +19917,11 @@
           <t>ФРС каже, що монетарна політика готова до економічних ризиків</t>
         </is>
       </c>
-      <c r="F325" s="11" t="inlineStr"/>
+      <c r="F325" s="11" t="inlineStr">
+        <is>
+          <t>ФРС каже, що монетарна політика готова до економічних ризиків Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G325" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -18679,7 +19975,11 @@
           <t>ОАЕ обговорює своп-лінію з США</t>
         </is>
       </c>
-      <c r="F326" s="11" t="inlineStr"/>
+      <c r="F326" s="11" t="inlineStr">
+        <is>
+          <t>ОАЕ обговорює своп-лінію з США Домен: валюта_фінанси Країна: ОАЕ</t>
+        </is>
+      </c>
       <c r="G326" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -18733,7 +20033,11 @@
           <t>Бавовна торгується змішано в понеділок</t>
         </is>
       </c>
-      <c r="F327" s="11" t="inlineStr"/>
+      <c r="F327" s="11" t="inlineStr">
+        <is>
+          <t>Бавовна торгується змішано в понеділок Домен: ціни_сировини</t>
+        </is>
+      </c>
       <c r="G327" s="11" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -18787,7 +20091,11 @@
           <t>Бессент закликає Китай до дипломатії щодо Ірану перед саміту</t>
         </is>
       </c>
-      <c r="F328" s="11" t="inlineStr"/>
+      <c r="F328" s="11" t="inlineStr">
+        <is>
+          <t>Бессент закликає Китай до дипломатії щодо Ірану перед саміту Домен: геополітика Країна: США, Китай, Іран</t>
+        </is>
+      </c>
       <c r="G328" s="11" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -18841,7 +20149,11 @@
           <t>ЄС виключив шкіру з закону про вирубку лісів</t>
         </is>
       </c>
-      <c r="F329" s="11" t="inlineStr"/>
+      <c r="F329" s="11" t="inlineStr">
+        <is>
+          <t>ЄС виключив шкіру з закону про вирубку лісів Домен: митниця_регуляторика Країна: ЄС</t>
+        </is>
+      </c>
       <c r="G329" s="11" t="inlineStr">
         <is>
           <t>митниця_регуляторика</t>
@@ -18899,7 +20211,11 @@
           <t>Аналіз ринку амінокислот у Великобританії</t>
         </is>
       </c>
-      <c r="F330" s="11" t="inlineStr"/>
+      <c r="F330" s="11" t="inlineStr">
+        <is>
+          <t>Аналіз ринку амінокислот у Великобританії Домен: ціни_сировини Країна: Великобританія</t>
+        </is>
+      </c>
       <c r="G330" s="11" t="inlineStr">
         <is>
           <t>ціни_сировини</t>
@@ -18957,7 +20273,11 @@
           <t>Moody's поліпшив прогноз для В'єтнаму</t>
         </is>
       </c>
-      <c r="F331" s="11" t="inlineStr"/>
+      <c r="F331" s="11" t="inlineStr">
+        <is>
+          <t>Moody's поліпшив прогноз для В'єтнаму Домен: валюта_фінанси Країна: В'єтнам</t>
+        </is>
+      </c>
       <c r="G331" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -19011,7 +20331,11 @@
           <t>Франція встановила дорожну карту сталості птахівництва до 2035</t>
         </is>
       </c>
-      <c r="F332" s="11" t="inlineStr"/>
+      <c r="F332" s="11" t="inlineStr">
+        <is>
+          <t>Франція встановила дорожну карту сталості птахівництва до 2035 Країна: Франція</t>
+        </is>
+      </c>
       <c r="G332" s="11" t="inlineStr">
         <is>
           <t>не_релевантно</t>
@@ -19065,7 +20389,11 @@
           <t>GBRf і Maritime Transport укладають новий контракт</t>
         </is>
       </c>
-      <c r="F333" s="11" t="inlineStr"/>
+      <c r="F333" s="11" t="inlineStr">
+        <is>
+          <t>GBRf і Maritime Transport укладають новий контракт Домен: логістика Країна: Великобританія</t>
+        </is>
+      </c>
       <c r="G333" s="11" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -19119,7 +20447,11 @@
           <t>Індонезія розширює торговельний профіцит до $3,32 млрд</t>
         </is>
       </c>
-      <c r="F334" s="11" t="inlineStr"/>
+      <c r="F334" s="11" t="inlineStr">
+        <is>
+          <t>Індонезія розширює торговельний профіцит до $3,32 млрд Домен: логістика Країна: Індонезія</t>
+        </is>
+      </c>
       <c r="G334" s="11" t="inlineStr">
         <is>
           <t>логістика</t>
@@ -19173,7 +20505,11 @@
           <t>Goldman Sachs прогнозує 30 можливих інтервенцій японської єни</t>
         </is>
       </c>
-      <c r="F335" s="11" t="inlineStr"/>
+      <c r="F335" s="11" t="inlineStr">
+        <is>
+          <t>Goldman Sachs прогнозує 30 можливих інтервенцій японської єни Домен: валюта_фінанси Країна: Японія</t>
+        </is>
+      </c>
       <c r="G335" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -19227,7 +20563,11 @@
           <t>Австралійський долар може ослабнути через РБА</t>
         </is>
       </c>
-      <c r="F336" s="11" t="inlineStr"/>
+      <c r="F336" s="11" t="inlineStr">
+        <is>
+          <t>Австралійський долар може ослабнути через РБА Домен: валюта_фінанси Країна: Австралія</t>
+        </is>
+      </c>
       <c r="G336" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -19281,7 +20621,11 @@
           <t>Трейдери стежать за двосторонніми ризиками на ринках</t>
         </is>
       </c>
-      <c r="F337" s="11" t="inlineStr"/>
+      <c r="F337" s="11" t="inlineStr">
+        <is>
+          <t>Трейдери стежать за двосторонніми ризиками на ринках Домен: валюта_фінанси</t>
+        </is>
+      </c>
       <c r="G337" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -19331,7 +20675,11 @@
           <t>АБР допомагає Тихоокеанським країнам від наслідків війни</t>
         </is>
       </c>
-      <c r="F338" s="11" t="inlineStr"/>
+      <c r="F338" s="11" t="inlineStr">
+        <is>
+          <t>АБР допомагає Тихоокеанським країнам від наслідків війни Домен: геополітика Країна: Тихоокеанські країни</t>
+        </is>
+      </c>
       <c r="G338" s="11" t="inlineStr">
         <is>
           <t>геополітика</t>
@@ -19385,7 +20733,11 @@
           <t>Тиждень: боротьба ФРС</t>
         </is>
       </c>
-      <c r="F339" s="11" t="inlineStr"/>
+      <c r="F339" s="11" t="inlineStr">
+        <is>
+          <t>Тиждень: боротьба ФРС Домен: валюта_фінанси Країна: США</t>
+        </is>
+      </c>
       <c r="G339" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>
@@ -19439,7 +20791,11 @@
           <t>Азійські облігаційні ринки показують рекордні обсяги випусків</t>
         </is>
       </c>
-      <c r="F340" s="11" t="inlineStr"/>
+      <c r="F340" s="11" t="inlineStr">
+        <is>
+          <t>Азійські облігаційні ринки показують рекордні обсяги випусків Домен: валюта_фінанси Країна: Азія</t>
+        </is>
+      </c>
       <c r="G340" s="11" t="inlineStr">
         <is>
           <t>валюта_фінанси</t>

</xml_diff>